<commit_message>
Regenerate exports with the updated corrigendum caveat
Reflects the confirmed-inaccessible corrigendum-access caveat (row 40,
Maisons et al. 2026) in both evidence-table.xlsx and
research-report.docx. QC-4 verified: xlsx row 40 carries the full
updated caveat text; docx contains the new wording at all 5 mentions
("Published Erratum" x5, updated phrasing present, none of the old
"content could not be verified" phrasing remains).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -2964,12 +2964,12 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Identified 3 distinct clinical phenotype clusters: (1) young males with GI/joint involvement and low renal risk; (2) middle-aged patients without GI involvement; (3) older patients with skin necrosis and high renal involvement/chronic renal failure — validated across two independent national cohorts.</t>
+          <t>Identified 3 distinct clinical phenotype clusters: (1) young males with GI/joint involvement and low renal risk; (2) middle-aged patients without GI involvement; (3) older patients with skin necrosis and high renal involvement/chronic renal failure — validated across two independent national cohorts. These numbers carry a confirmed, unresolved corrigendum-access caveat — see Notes column.</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>CAVEAT: a published corrigendum exists (DOI 10.1016/j.ejim.2026.107059, PMID 42457434) whose content could not be verified (no abstract, full text inaccessible with available tools). The numeric/cluster findings above have NOT been checked against the corrigendum — treat with caution until the corrigendum text is reviewed (see source record for full resolution rationale; escalated to orchestrator for literature-scout follow-up). Otherwise a notable methodological strength: independent two-country validation of the clustering result.</t>
+          <t>CAVEAT (updated 2026-09-13, following `literature-scout`'s Run 19 follow-up): a published corrigendum (Erratum) exists for this article — PMID 42457434, DOI 10.1016/j.ejim.2026.107059, Eur J Intern Med 151:107059. Its *existence* and formal "Published Erratum" classification (as opposed to a retraction or expression of concern) are now confirmed. Its *substantive content* — what specific figure, cluster definition, or number was corrected — remains inaccessible: an exhaustive 10-step verification attempt (PubMed metadata, PMC lookup, DOI resolution, direct ScienceDirect/PDF fetch [403 Forbidden], Crossref, Unpaywall, EuropePMC, reformulated web searches, and the EFIM reprint page — full detail in `sources/search-log.md` Run 19 and the dated addendum in this study's source-record Verification notes) found every full-text path either paywalled, a bare redirect/metadata stub, or abstract-empty. This upgrades the caveat from "not yet checked" to "actively verified as currently inaccessible despite exhaustive effort" — a materially stronger disclosure, though the underlying uncertainty about whether/how the cluster findings above (n=260/n=208, phenotype definitions) were affected by the correction is unchanged and genuinely unresolved. RETAINED as Included (tier 4), not downgraded or excluded, because (a) the confirmed "Published Erratum" classification typically denotes correction of a discrete error rather than invalidation of the study, and (b) the independent two-country (French/Slovenian) validation of the clustering result is a structural methodological strength unlikely to be nullified by a typical erratum-level correction. `research-writer` must present this row's specific figures with this caveat explicitly stated (not as settled numbers) and must not treat the exhausted verification effort as having resolved the uncertainty — it only rules out further easy resolution; full resolution would require institutional/subscription access to ScienceDirect or direct correspondence with the journal/authors. Otherwise a notable methodological strength: independent two-country validation of the clustering result.</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate exports with the Gandolfini confidence upgrade
Reflects row 15's LOW-to-MODERATE confidence upgrade and the
secondary-source-derived ~n=10/no-benefit description in both
evidence-table.xlsx and research-report.docx. QC-4 verified: xlsx row
15 carries the updated MODERATE-CONFIDENCE notes and PMC12630289
citation; docx contains the updated wording at all mentions with none
of the old low-confidence-only phrasing remaining.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -1394,32 +1394,32 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Research letter / small case series (tier-7 carve-out; LOW-CONFIDENCE classification — see file header and source record)</t>
+          <t>Research letter / small case series (tier-7 carve-out; MODERATE-CONFIDENCE classification, upgraded 2026-09-13 from LOW — see file header judgment call #1 and source record)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not extractable from available text (title indicates recurrent IgAN after kidney transplantation; no patient count or demographic detail available)</t>
+          <t>Per a secondary/citing source (PMC12630289), NOT independently verified against Gandolfini et al.'s own text: approximately 10 kidney-transplant recipients with recurrent IgAN. Gandolfini et al.'s own primary text remains unread (inaccessible through 11 independent paths — see source record); this population description is a citing-paper's paraphrase, not a direct extraction from the primary source.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>TRF-budesonide (Nefecon) in recurrent IgAN after kidney transplantation — a population not covered by NefIgArd's (rows 13–14) inclusion criteria</t>
+          <t>TRF-budesonide (Nefecon) in recurrent IgAN after kidney transplantation — a population not covered by NefIgArd's (rows 13–14) inclusion criteria. Per the same secondary source, patients were already on background transplant corticosteroids (not independently verified).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Not extractable from available text</t>
+          <t>Not extractable from available text (per the citing source's description this appears to be a single-arm case series; no formal comparator arm implied, but this is inferred from the secondary source, not confirmed)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>NOT EXTRACTABLE FROM AVAILABLE TEXT. No abstract is available via PubMed (confirmed via `get_article_metadata`); full text is paywalled (ScienceDirect returned HTTP 403) and no PMC ID exists. Only the title and bibliographic context could be used; no numeric findings are reported here to avoid fabrication.</t>
+          <t>Per a secondary/citing source (PMC12630289, Journal of Nephrology 2025), NOT independently verified against Gandolfini et al.'s own text: "Gandolfini et al. analyzed 10 patients receiving targeted-release budesonide after kidney transplantation and found no benefit from therapy, concluding that there was no additional effect as patients were already on corticosteroids to prevent allograft rejection" — the citing paper further notes a different (whole-colon-release) formulation and a lower dose/shorter duration than its own case. This is a citing-paper's paraphrase of Gandolfini et al.'s content, not a verbatim quote or direct extraction from Gandolfini et al.'s own text (which remains inaccessible through 11 independent paths — see source record). It is uncorroborated by a second independent citing source (PMC12638209 cites the same DOI only generically, without repeating this detail, and lists a non-matching author string — flagged as a likely citation error in that second source, not as contradicting evidence). No numeric findings are extracted directly from Gandolfini et al.'s own text; treat the n=10/"no benefit" description as a low-confidence secondary-source lead only, not a confirmed finding, and do not cite it with the same weight as any directly-extracted row in this table.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>LOW-CONFIDENCE INCLUSION. PubMed classifies this article as "Letter"/"Comment"; evidence-reviewer resolved it as a probable data-bearing research letter rather than a non-data commentary based on title pattern and Kidney International's correspondence-format conventions (full rationale in source record), but this could NOT be confirmed from any available text. If full text later becomes available and shows this is pure commentary with no original data, this row should be removed/reclassified to Background/Context — flagged in handoff summary.</t>
+          <t>MODERATE-CONFIDENCE INCLUSION (upgraded 2026-09-13 from LOW; see file-header judgment call #1 and source record's dated confidence-update note for full rationale). PubMed classifies this article as "Letter"/"Comment"; evidence-reviewer's classification as a data-bearing research letter (tier-7 carve-out) rather than a non-data commentary is now supported by two independent, mutually-reinforcing indirect signals — a paired "authors reply" from NefIgArd's own senior investigators (Barratt &amp; Rovin), and a citing paper's specific-n paraphrase — but is still not confirmed against Gandolfini et al.'s own primary text, which remains inaccessible through 11 independent paths (PubMed, PMC, DOI resolution, publisher site, Crossref, Unpaywall, EuropePMC, Semantic Scholar, corresponding-author's institutional repository, ResearchGate — a confirmed dead end, comparable to the Maisons corrigendum situation in row 40). The n=10/"no benefit" description is sourced from a single, uncorroborated citing paper (PMC12630289), not from Gandolfini et al.'s own text — evidence-reviewer judges this secondary-source paraphrase to be meaningfully different from a direct primary-text extraction (it is a third party's characterization, subject to that party's own potential misreading, selective emphasis, or error, and cannot be checked against Gandolfini et al.'s actual reported methodology, statistics, or exact wording), so it is recorded here ONLY under this explicit secondary-source label. Reviewer-identified: the citing paper's own explanation for the null result (different formulation/lower dose/shorter duration) is that citing author's own interpretation, not an author-stated limitation of Gandolfini et al. — do not attribute it to Gandolfini et al. as such. If full text later becomes available and confirms, contradicts, or refines this description, this row must be updated accordingly (flagged in handoff summary).</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 44-52)
evidence-table.xlsx: 52 Included Studies rows (was 43), 5
Background-Context rows, 1 Excluded row, regenerated directly from
evidence-table.md. research-report.docx: regenerated from
research-report.md, now 53 references (48 primary + 5 background).

QC-4 verified: xlsx row count matches; docx contains all 8 new paper
citations plus 53 correctly-targeted DOI hyperlinks.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3166,6 +3166,564 @@
       <c r="L44" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.1097-MD.0000000000036521.md (../sources/papers/10.1097-MD.0000000000036521.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Wu et al. 2026 (C1GALT1 B-cell knockout mouse)</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Kidney International</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Preclinical mechanistic study, in vivo mouse model (tier 6)</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Humanized IGHA1 knock-in mouse with B cell-specific c1galt1 deletion, studied under physiological conditions and following inflammatory stimulation (Lactobacillus casei cell wall extract + complete Freund's adjuvant); plus a passive-transfer mouse model comparing IgA1 sourced from human serum, ileocecal mucus, and myeloma patients</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Wild-type (c1galt1-intact) IGHA1 knock-in mice, physiological vs. inflammatory-stimulation conditions; comparison across IgA1 tissue-of-origin in the passive-transfer model</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>None tested as an intervention (genetic/mechanistic model); no drug/therapy evaluated</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>B cell-specific c1galt1 deletion markedly elevated circulating Gd-IgA1 both at baseline and after inflammatory stimulation, and impaired B cell development/systemic and mucosal IgA production — but glomerular IgA deposition remained limited and was NOT substantially enhanced by inflammatory stimulation despite the markedly elevated Gd-IgA1. In the passive-transfer model, mucosa (ileocecal)-derived IgA1 from IgAN patients caused significantly stronger mesangial deposition than serum- or myeloma-derived IgA1, despite similar or lower Gd-IgA1 content. Authors conclude Gd-IgA1 is "a correlate of mucosal immune activation rather than a direct pathogenic driver," with tissue origin/immune context as the more likely determinant of deposition/pathogenicity.</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Reviewer-identified conflict/nuance: this dissociation between Gd-IgA1 elevation and glomerular deposition nuances the Gd-IgA1-centered "multiple-hit" pathogenic model underlying several complement- and BAFF/APRIL-targeted therapies elsewhere in this table (rows 16–19, 20–23, 27–28) and the mucosal-origin findings in rows 29–30 — flagged as an unresolved mechanistic tension for `research-writer` to represent, not resolve. Preclinical only; exact group sample sizes not stated in the available abstract text (full text paywalled — WebFetch redirect blocked). Academic, multi-institution (China/UK/US) collaboration.</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.kint.2026.02.034 / PMID 41905596</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.kint.2026.02.034.md (../sources/papers/10.1016-j.kint.2026.02.034.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Gentile et al. 2024</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Kidney Int Reports</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Case-control mechanistic/immunophenotyping study with independent validation cohort (tier 6; see file header judgment call #8)</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>66 patients with biopsy-proven IgAN and 30 healthy controls (Mount Sinai NYC + Hospital de Navarra, Spain); CyTOF subset n=35 IgAN/14 controls; validation cohort (NURTuRE study, whole-blood RNAseq): 179 IgAN, 140 minimal change disease, 91 healthy controls</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>None (observational; serum IgA/Gd-IgA1/BAFF/APRIL, stool IgA-coated bacteria, CyTOF immunophenotyping of B cells and unconventional T cells)</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Healthy controls; minimal change disease as disease control in the validation cohort</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>IgAN patients had significantly higher circulating total IgA and Gd-IgA1, and higher APRIL (p=0.032, not BAFF, p=0.571) vs. controls; higher IgA (p=0.022) and Gd-IgA1-positive (p=0.033) gut bacteria (no difference in IgG-coated bacteria, p=0.089). CyTOF: class-switched memory (p=0.022) and double-negative (p=0.041) B cells significantly higher; MAIT cells (p=0.0017) and γδ T cells (p=0.0014) significantly lower; CD4-CD8- NKT cells significantly higher (p=0.005) in IgAN vs. controls. MAIT cell reduction (via SLC4A10 expression) was validated in the independent 179-patient NURTuRE cohort (p&lt;0.0001) and was IgAN-specific (not seen comparing minimal change disease to controls, p=0.24).</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Authors note an apparent contrast with an RCT showing no efficacy of rituximab (B cell depletion) in IgAN, speculating peripheral B cell depletion doses may not adequately deplete gut-mucosal B cells — an interpretive point relevant to rows 22–23 (atacicept/telitacicept) and the wider BAFF/APRIL-targeted-therapy rationale. Two-site discovery cohort with independent multi-site validation is a design strength. All authors declared no competing interests.</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.ekir.2024.11.007 / PMID 39990906</t>
+        </is>
+      </c>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.ekir.2024.11.007.md (../sources/papers/10.1016-j.ekir.2024.11.007.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Xiong et al. 2024 (rituximab in IgAVN)</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Clinical and Experimental Medicine</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review of the published literature, pooled patient-level case data (tier 1; see file header judgment call #7 re: underlying case-report-level evidence)</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>41 patients with biopsy-proven IgA vasculitis nephritis pooled from 28 published articles (multi-database search through Dec 29, 2023); median age 28y (range 14–49), 48.8% female, both adults and children</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Rituximab (RTX), predominantly as add-on therapy (37/41) after glucocorticoids (97.5%) ± other immunosuppressants (60.0%); 3/41 as monotherapy</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>None (single-arm pooled case-level data; pre-/post-RTX comparison; pediatric-vs-adult subgroup comparison)</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Remission rate 92.7% (38/41); complete remission 46.3% (19/41). Children achieved complete remission significantly more often than adults (76.9% [10/13] vs. 32.1% [9/28], p=0.017). Haematuria fell from 84.8% (28/33) to 12.1% (4/33) (p&lt;0.001); proteinuria/glucocorticoid-use/cutaneous/abdominal/joint manifestations all significantly improved (p&lt;0.001 to p=0.003). eGFR&lt;60 mL/min/1.73m² fell from 42.3% (11/26) to 30.7% (8/26), NOT statistically significant (p=0.425). 4.9% (2/41) non-response; 2.4% (1/41) death (adult). No serious adverse events reported.</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: entirely derived from published case reports/series — inherent publication bias likely overestimating RTX efficacy; highly diverse baseline data; cannot standardize follow-up timepoints across sources; authors explicitly call for prospective controlled studies. Reviewer-identified: no comparator/control arm — causal attribution of remission to RTX vs. concurrent glucocorticoids/immunosuppressants (in the 37/41 add-on cases) is confounded. Paper itself contrasts its positive IgAVN signal with a cited RCT showing no significant renal-function/proteinuria benefit of rituximab in (non-vasculitic) IgAN — an unexplained IgAN-vs-IgAV discrepancy the authors flag but do not resolve. Cross-reference/tension: read alongside row 38 (Rohner et al., null finding on second-line-regimen superiority in IgAVN) and row 1 (Cochrane IgAV review's low/moderate-certainty null findings) — this review's positive RTX signal sits in tension with that broader sparse/null high-quality IgAVN treatment evidence base; presented here as an unresolved conflict, not reconciled.</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s10238-024-01461-6 / PMID 39249581</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s10238-024-01461-6.md (../sources/papers/10.1007-s10238-024-01461-6.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Damman et al. 2022</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Molecular Immunology</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective case-control immunofluorescence/mechanistic study (tier 6; see file header judgment call #8)</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>17 patients with IgA-vasculitis skin biopsies vs. 25 non-IgAV control skin biopsies (retrospective)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>None (observational) — direct immunofluorescence for IgA, IgG, IgM, C1q, C4d, properdin, MBL, FCN2, MASP1/3, MASP2, C3c in cutaneous vessels</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Non-IgAV control biopsies (n=25); internal comparison of complement-factor deposition against IgAVN development and treatment response</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Properdin positive in 82% of IgAV cases (alternative pathway); C4d positive in 88% (classical and/or lectin pathway) though C1q positive in only 12% (suggesting lectin- rather than classical-pathway-driven C4d); MBL positive 47%, MASP1/3 53%, MASP2 6%; FCN2 negative. MASP1/3 deposition significantly higher in IgAV vs. non-IgAV controls. NULL FINDING: no significant association between complement-pathway activation and progression to IgAVN or response to therapy — authors explicitly state "it is unlikely that intervention in complement activation will lead to a better clinical course of the disease," tempering their own paper's "new target for therapy" framing.</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: first demonstration of lectin/alternative pathway activation specifically in cutaneous IgAV; explicitly caution that no clinical-course/treatment-response association was found. Reviewer-identified: small retrospective cohort (17 vs. 25); cross-sectional immunofluorescence design cannot establish causality or predict clinical course. Cross-reference row 3 (Ștefan et al., MEST-C/complement systematic review, renal focus) and rows 16–19/27–28 (complement-targeted IgAN therapies) — this study's null clinical-correlation finding is a relevant caveat specific to cutaneous/systemic IgAV manifestations, distinct from the renal (IgAVN) complement evidence in row 3.</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.molimm.2022.01.011 / PMID 35121432</t>
+        </is>
+      </c>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.molimm.2022.01.011.md (../sources/papers/10.1016-j.molimm.2022.01.011.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Batista-Liz et al. 2023</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>International Journal of Molecular Sciences</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>Case-control genetic-association study (tier 6; see file header judgment call #8)</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>381 unrelated Caucasian IgAV patients (multi-center Spain) vs. 997 unrelated ethnically/sex-matched healthy controls (National DNA Bank Repository, Salamanca); subgroups by age at onset (≤20y vs. &gt;20y) and by GI/renal (nephritis) manifestation status</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>None (observational) — genotyping of 7 mucosal immune defence polymorphisms (ITGAM/ITGAX rs11150612/rs11574637, VAV3 rs17019602, CARD9 rs4077515, DEFA1/DEFA3 rs2738048/rs10086568, FUT2 rs2412971), previously reported as IgAN susceptibility loci</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Healthy controls; IgAVN subgroup vs. controls; IgAV subgroups by age-of-onset and GI/renal-manifestation status</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>NULL/NEGATIVE FINDING (explicitly represented per source-record instruction and research-question.md's evidence-gap requirement): no statistically significant differences in genotype, allele, or haplotype frequencies for any of the 7 polymorphisms between the overall IgAV cohort and controls, nor between the IgAVN subgroup and controls, nor across age-of-onset or GI/renal-manifestation strata. Authors conclude these established IgAN risk loci do NOT represent genetic risk factors for IgAV susceptibility or severity, and suggest this reinforces IgAV and IgAN as potentially genetically distinct entities despite shared clinical/pathologic features.</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: largest Caucasian IgAV genetic cohort assessed to date for these variants; consistent with the same group's prior null finding for a related mucosal-defence gene in IgAV; authors suggest future work focus on complement-pathway/IgA-glycosylation loci instead. Reviewer-identified: single-ethnicity (Caucasian) cohort limits generalizability; a null finding at this sample size still cannot rule out small-effect-size associations (power caveat not addressed in the available text). Notable evidence-gap/divergence finding: contrasts with the IgAN literature (where these same loci ARE risk-associated, per the paper's own framing) — an explicit IgAN-vs-IgAV genetic-divergence data point for `research-writer` to represent, not smooth over.</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr">
+        <is>
+          <t>10.3390/ijms241713063 / PMID 37685869</t>
+        </is>
+      </c>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.3390-ijms241713063.md (../sources/papers/10.3390-ijms241713063.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Demir et al. 2023</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Diagnostics (Basel)</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>Cross-sectional untargeted plasma proteomics study (tier 6; see file header judgment call #8)</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>37 active pediatric IgAV patients (24F/13M, mean age 8.77±3.54y) and 5 age-matched healthy children (3M/2F, mean age 8.91±4.07y), Turkey; none of the IgAV patients had renal involvement at diagnosis or at 1-year follow-up</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>None (observational) — nano-LC-MS/MS untargeted plasma proteomic profiling, pre-treatment</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Healthy pediatric controls (n=5)</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Of 348 quantifiable proteins, 20 were significantly differentially expressed (15 up, 5 down) vs. controls. KEGG/Reactome analysis identified complement and coagulation cascades as most enriched. Lectin-pathway marker MASP1 was 13.46-fold higher; alternative-pathway CFB 1.72-fold higher; terminal-pathway C9 1.99-fold higher; SERPINA5 (a MASP1/2 inhibitor) 3.7-fold lower. Additional alterations in vascular-adhesion (cadherin-5, IGFALS) and coagulation (F13A1, 5-fold decrease) proteins. Authors conclude findings support lectin and alternative (not classical) complement-pathway activation in IgAV — converging with rows 3 and 47's complement-pathway findings.</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: "the major limitation of this study is the small number of the groups" — explicitly framed as a first-step, hypothesis-generating study requiring targeted-proteomic validation. Reviewer-identified: control group of n=5 vs. 37 cases is a severe case:control imbalance (flagged by literature-scout for this appraisal) substantially limiting statistical power and increasing false-positive/negative risk — treat as exploratory/hypothesis-generating only. No IgAV patients in this cohort had renal involvement, so findings cannot be directly extrapolated to IgAVN specifically.</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>10.3390/diagnostics13101729 / PMID 37238213</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.3390-diagnostics13101729.md (../sources/papers/10.3390-diagnostics13101729.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Mayer-Hain et al. 2022</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>The Journal of Immunology</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Mixed human + murine mechanistic/immunological study (tier 6)</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Human IgAV patients (serum/PMN and skin-biopsy samples during acute flares; exact n not extractable from available text) plus a murine immune-complex vasculitis model (including myeloperoxidase-knockout mice); in vitro neutrophil (PMN) functional assays and a flow system mimicking postcapillary venule conditions</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Surface-IgA-negative PMNs (post-flare); IgAV patients without flares vs. during flares; wild-type vs. MPO-knockout/NET-inhibited mice</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>IgA-immune-complex (IgA-IC) binding to circulating PMNs; FcαRI blockade; myeloperoxidase (MPO) knockout; NET-formation inhibition</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>During acute IgAV flares, serum IgA-IC levels and IgA-IC binding to circulating PMNs were elevated, priming PMNs and lowering the NETosis threshold (significantly higher NET release vs. IgA-negative PMNs post-flare). FcαRI blockade abolished this effect; complement was NOT essential for this mechanism — a notable finding distinguishing this pathway from the complement-centric IgAV mechanisms in rows 3, 47, and 49. Marked NETosis required PMN adhesion to activated endothelial cells; IgA-IC binding enhanced PMN-endothelial tethering and NET-mediated endothelial injury; NETs were visualized near endothelial cells/IgA-coated PMNs in patient tissue. In vivo, NET-formation inhibition and MPO knockout significantly reduced vessel damage in the murine model.</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated framing: IgA-IC deposition alone is "mandatory but not sufficient" for IgAV; systemic neutrophil priming/NETosis proposed as an additional necessary mechanistic step. Reviewer-identified: exact human sample size and specific p-values/fold-changes not extractable from available text — full text was paywalled/inaccessible (no PMCID; WebFetch on the journal URL returned only a loading placeholder); extraction is abstract-level only. Combines human correlative and murine causal (knockout) evidence — a design strength. Its complement-independent finding should be read as a complementary (not necessarily contradictory) pathway alongside the complement-centric findings in rows 3, 47, 49, not merged with them.</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr">
+        <is>
+          <t>10.4049/jimmunol.2100924 / PMID 35985788</t>
+        </is>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.4049-jimmunol.2100924.md (../sources/papers/10.4049-jimmunol.2100924.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Lin et al. 2025 (Dioscin/IL-6-JAK2-STAT3)</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>BMC Nephrology</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Mixed human PBMC case-control + murine model + in vitro mechanistic study (tier 6)</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>68 IgAN patients (biopsy-confirmed adults) vs. 16 age/sex-matched healthy controls (PBMC qRT-PCR); Balb/c mouse IgAN model (mucosal immunization, n=6/group for histology/IF/IHC endpoints); DAKIKI human B-lymphocyte cell line in vitro</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Healthy controls (human); saline-treated normal-control and untreated Model-group mice; untreated/vehicle DAKIKI cells</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Dioscin (DIO), active compound of Yiqi Qingjie Formula (Traditional Chinese Medicine) — 0.06 g/kg intragastric in mice, 0.25–1.0 µg/mL in vitro; IL-6 (12.5–100 ng/mL) used to model Gd-IgA1 hypersecretion in DAKIKI cells</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>mRNA levels of IL-6R, gp130, and STAT3 were significantly upregulated in PBMCs from IgAN patients vs. controls. In mice, DIO treatment visibly reduced mesangial IgA deposition, mesangial proliferation/matrix expansion, and Peyer's-patch lymphocyte hyperplasia, and suppressed p-JAK2/p-STAT3/STAT3 in Peyer's patches (n=6/group; qualitative/IHC endpoints, no group-level p-values given for histology). In DAKIKI cells, IL-6 (25 ng/mL) increased Gd-IgA1/IgA secretion and downregulated C1GalT1/Cosmc; DIO (1.0 µg/mL) dose-dependently suppressed IL-6-induced proliferation, IgA/Gd-IgA1 secretion (20.8% suppression at 1.0 µg/mL), JAK2/STAT3 mRNA upregulation, and STAT3 phosphorylation (significance denoted *p&lt;0.05/p&lt;0.01/*p&lt;0.001; exact p-values beyond these thresholds not extractable from available text).</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated limitations (explicit): (1) DIO is currently approved only as adjuvant therapy for coronary heart disease/angina, not IgAN, so could not be administered to enrolled patients, limiting the link between clinical PBMC findings and the animal/cell experiments; (2) small IgAN cohort limited comprehensive pathway-regulator assessment; (3) mice cannot produce Gd-IgA1 due to species-specific characteristics, so no direct in vivo evidence of DIO inhibiting Gd-IgA1 was obtained; (4) no JAK2/STAT3 pathway-inhibition or gene-knockout experiments were performed to directly validate the target. Reviewer-identified: single-center (China); preclinical/mechanistic evidence only, no clinical efficacy/safety data for DIO in IgAN patients. Complements row 33 (Lang et al., Rehmannia glutinosa/Catalpol) as another TCM-derived preclinical mechanistic candidate — not to be conflated with clinical-grade evidence.</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr">
+        <is>
+          <t>10.1186/s12882-025-04614-1 / PMID 41402741</t>
+        </is>
+      </c>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1186-s12882-025-04614-1.md (../sources/papers/10.1186-s12882-025-04614-1.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Huang et al. 2025 (SOCS1/TLR9/MyD88)</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Immunologic Research</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Mixed mouse model + cell line + human bioinformatics/immunofluorescence mechanistic study (tier 6)</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>IgAN mouse model (strain/species detail not extractable from available abstract text); IgA1-secreting DAKIKI human B-lymphocyte cell line; human renal tissue and PBMC samples from IgAN vs. non-IgAN patients (exact n not extractable from available text) plus public bioinformatics dataset GSE35487</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Non-IgAN patients/controls (bioinformatics/IF comparison); untransfected/control DAKIKI cells; comparison across SOCS1-overexpression vs. knockdown vs. MyD88-knockdown conditions</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>SOCS1 overexpression/knockdown in DAKIKI cells; MyD88 knockdown; CpG-ODN (TLR9 ligand) stimulation; in vivo SOCS1 manipulation in the mouse model (delivery method not extractable from available text)</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>SOCS1 expression was suppressed in renal tissue and PBMCs of IgAN patients vs. controls, consistent with the public GSE35487 dataset. C1GALT1 in PBMCs was decreased and positively correlated with SOCS1, while TLR9 and MyD88 were increased and negatively correlated with SOCS1 (exact correlation coefficients/p-values not extractable from available text). In vitro, SOCS1 overexpression inhibited IgA1/Gd-IgA1 secretion and TLR9 expression; knockdown had the opposite effect. MyD88 knockdown reversed CpG-ODN-induced Gd-IgA1/IgA1 overproduction and C1GALT1 reduction, supporting a SOCS1-TLR9-MyD88-C1GALT1 regulatory axis. In vivo, SOCS1 reduced aberrantly glycosylated IgA-IgG immune complexes and IL-6, reduced glomerular IgA/IgG/C3 deposition and mesangial proliferation, and alleviated renal injury.</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Not extractable from available text: exact sample sizes for the mouse model and human PBMC/renal-tissue comparison, specific statistical values, and the authors' own stated limitations section — full text was not accessible (no PMCID; WebFetch attempts on the DOI/publisher redirect were blocked), so this row is abstract-level extraction only. Reviewer-identified: preclinical/mechanistic study only (mouse + cell line + retrospective bioinformatics) — no clinical efficacy or human interventional data; single abstract-level source limits appraisal of methodological rigor (e.g., randomization, blinding, sample-size justification) — treat as hypothesis-generating.</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s12026-025-09669-8 / PMID 40759858</t>
+        </is>
+      </c>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s12026-025-09669-8.md (../sources/papers/10.1007-s12026-025-09669-8.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (row 53)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3724,6 +3724,68 @@
       <c r="L53" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.1007-s12026-025-09669-8.md (../sources/papers/10.1007-s12026-025-09669-8.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Kumaş et al. 2026 (sarsasapogenin)</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>The FASEB Journal</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Preclinical mechanistic study, controlled in vivo rat model, randomized allocation with blinded outcome assessment (tier 6 — mechanistic/preclinical animal model relevant to pathogenesis and a novel therapeutic target)</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Male Sprague-Dawley rats; experimental IgAN induced via sequential BSA (intragastric)/CCl4 (subcutaneous)/LPS (IV) administration over 9–12 weeks; 17 rats underwent induction (3 sacrificed for model-validation only, excluded from final analysis) + 14 healthy rats; final analysis n=7/group across 4 groups (Control, SAR-only, IgAN+vehicle, IgAN+SAR), total n=28; single-center (Dokuz Eylul University, Turkey)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Sarsasapogenin (SAR), a steroidal sapogenin natural compound, 60 mg/kg/day intragastric gavage, weeks 7–12 (6-week treatment course)</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Vehicle (1% CMC-Na) in disease and healthy groups (2×2 design: Control, SAR-only, IgAN+vehicle, IgAN+SAR)</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Model validation: mesangial IgA deposition confirmed by IHC, significantly higher in IgAN group vs. control/SAR (p&lt;0.0001); SAR markedly attenuated IgA accumulation in IgAN+SAR (exact % values presented only graphically in figures, not printed in text). Renal function/proteinuria: urinary protein rose progressively in IgAN, peaking week 10; SAR significantly reduced proteinuria at weeks 10 and 12; serum urea/creatinine significantly higher in IgAN vs. control/SAR, significantly reduced by SAR (not fully normalized to healthy levels); SAR alone had no effect on renal parameters in healthy animals (exact numeric values/p-values for these panels given only as significance bands in figure legends: *p&lt;0.05 to p&lt;0.0001, not as printed values in running text). Inflammation/fibrosis markers: serum IL-6 significantly elevated in IgAN, significantly reduced by SAR; serum TNF-α showed only modest, apparently non-significant differences across groups; TGF-β1, SMAD3, and PDGF significantly elevated in IgAN vs. healthy groups, attenuated by SAR (most pronounced for TGF-β1/SMAD3); glomerular fibronectin and α-SMA (IHC) significantly increased in IgAN, significantly reduced by SAR though remaining above healthy levels. Masson's trichrome showed no significant collagen deposition in any group — authors interpret this as early fibrogenic activation preceding overt fibrosis, not established fibrosis. Oxford MEST-C: IgAN group had significantly higher frequencies of M1, E1, S1, T1, and C1 vs. control/SAR (Fisher's exact, *p&lt;0.05/*p&lt;0.001); SAR significantly reduced M1 and E1 prevalence specifically (from 100% in untreated IgAN to 28.6% in IgAN+SAR); reductions in S1, T1, and C1 with SAR were smaller and, per the authors' own discussion, non-significant. Podocyte integrity: TEM showed focal foot-process effacement in IgAN, partially preserved architecture in IgAN+SAR; nephrin and podocin (IHC and Western blot) significantly reduced in IgAN, significantly increased by SAR (partial restoration, remaining below healthy-group levels). No mortality in any group.</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated limitations (paraphrased from the paper's own "Limitations of the Study" section): (1) 12-week experimental duration captures only the early-to-moderate disease stage and precludes evaluating SAR's long-term efficacy or potential late-stage toxicity; (2) sample sizes, while "statistically sufficient to confirm significant associations," would benefit from larger cohorts for generalizability; (3) a definitive causal mechanism for the TGF-β1/SMAD3 and IL-6 pathway modulation remains unestablished absent gene-knockout or receptor-blocking experiments; (4) rodent-human physiological/metabolic differences necessitate caution when extrapolating the Oxford MEST-C-scored preclinical findings to human clinical settings. Reviewer-identified: single-center study (Dokuz Eylul University, Turkey), n=7/group is a small (though preclinical-typical) sample; academic funding only (Dokuz Eylul University Scientific Research Project Foundation, Grant TSG-2023-3262) with an explicit no-conflicts-of-interest declaration — lower industry-bias risk than several sponsor-funded rows elsewhere in this table. Notable methodological strengths relative to other tier-6 rows in this table: computer-generated randomization to groups, and histopathological/immunohistochemical/quantitative analyses performed by investigators blinded to group allocation (including two independently blinded pathologists for MEST-C scoring) — blinding is not reported for several other preclinical rows (e.g., rows 33, 51, 52). A limitation of this extraction: most quantitative effect sizes (percentages, fold-changes) are presented only graphically in the paper's figures rather than as printed numeric values in the running text; this row therefore records directionality and statistical-significance bands accurately but cannot report exact magnitudes beyond the one figure explicitly stated in text (M1/E1 prevalence 100%→28.6%). No conflict identified with other included studies' central findings; complements other natural-compound/TCM-derived preclinical rows targeting overlapping inflammatory/TGF-β-SMAD pathways (row 33, Rehmannia glutinosa/Catalpol in IgAV mice; row 51, Dioscin in IgAN) with a consistent, non-contradictory direction of effect, and adds podocyte-ultrastructure (TEM) evidence not present in those rows.</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr">
+        <is>
+          <t>10.1096/fj.202602487R / PMID 42698355 (PMCID PMC13545654)</t>
+        </is>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1096-fj.202602487R.md (../sources/papers/10.1096-fj.202602487R.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 54-57)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3786,6 +3786,254 @@
       <c r="L54" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.1096-fj.202602487R.md (../sources/papers/10.1096-fj.202602487R.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Wang et al. 2026 (ELISA Poly-IgA)</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Nephrology</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective two-center diagnostic-accuracy cohort with defined comparator groups (tier 4)</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Clinical samples from two independent centers: healthy controls, patients with IgA nephropathy (IgAN), and patients with non-IgAN kidney disease (nKD: membranous nephropathy, FSGS, other biopsy-confirmed glomerular disease); exact per-group sample sizes not extractable from available text (abstract-level only — full text paywalled)</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>ELISA-based test kit for circulating polymeric IgA immune complexes (Poly-IgA) as a candidate diagnostic biomarker</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Non-IgAN kidney disease (nKD) patients and healthy controls</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Analytical validation: limit of blank (LOB) 10 U/mL, recovery 85–105%, linear range 15.63–500 U/mL. Diagnostic performance (ROC analysis, retrospective clinical samples): AUC 0.87; at optimal cutoff 75.6 U/mL, sensitivity 82.7%, specificity 76.0%, overall accuracy 78.0% for differentiating IgAN from nKD.</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: specificity of 76% is "insufficient to replace kidney biopsy as the diagnostic gold standard"; authors explicitly flag the "relatively small sample size" and call for "prospective multicenter studies in larger and more diverse populations." Reviewer-identified: full text is paywalled (Dustri/Clinical Nephrology publisher site redirect loop confirmed; no PMCID) — extraction is abstract-level only, so exact per-group sample sizes, precision/reproducibility statistics beyond LOB/recovery/linear range, and any conflict-of-interest/funding disclosure are not extractable from available text. Diagnostic (not therapeutic) evidence — complements but does not overlap with the Gd-IgA1/mucosal-biomarker mechanistic rows elsewhere in this table (rows 29–30, 45).</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr">
+        <is>
+          <t>10.5414/CN111934 / PMID 42770490</t>
+        </is>
+      </c>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.5414-CN111934.md (../sources/papers/10.5414-CN111934.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Pan et al. 2026 (China IgAN real-world cohort)</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>BMJ Open</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective regional electronic-health-record cohort study (tier 4)</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>978 adult biopsy-proven primary IgAN patients, Yinzhou District, Ningbo City, China; identification period Jan 2015–Jun 2023; median age 43y, 52.03% female; 85.94% Lee grade III–V; 98.85% M1, 77.78% E1, 78.93% S1 (Oxford classification)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>RAAS inhibitors, SGLT2 inhibitors, corticosteroids, nonsteroidal immunosuppressants, traditional Chinese medicine (TCM) — treatment patterns tracked pre-biopsy, at initial treatment, and during entire follow-up (2016–2023 temporal trends)</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Internal reference-group comparisons (proteinuria-at-biopsy and time-averaged-proteinuria strata, vs. &lt;0.5 g/day reference)</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Composite renal events (ESKD, 40% eGFR decline, creatinine doubling, all-cause mortality) in 6.65% (65/978) over median 2.83-year follow-up; 5-year event-free probability 90.5% (95% CI 88.2–92.9%). eGFR-slope regression: proteinuria 0.5–1 g/day at biopsy β=−5.14 (95% CI −9.47 to −0.83, p=0.024); 1–2 g/day β=−5.90 (p=0.007); 2–3 g/day β=−6.36 (p=0.015). Composite-event hazard ratios (vs. &lt;0.5 g/day at biopsy): ≥3 g/day HR 3.44 (95% CI 1.42–8.36, p=0.006); time-averaged proteinuria ≥3 g/day HR 4.09 (95% CI 1.80–9.29, p=0.001). RAASi use rose to 91.49% during follow-up; SGLT2i uptake rose from negligible to 14.66% overall (17.14% by 2023); corticosteroid use declined from 36.62% (2016) to 16.49% (2023) while nonsteroidal immunosuppressant use rose to 31.89% by 2023. 41.80% achieved time-averaged proteinuria &lt;0.5 g/day; 58.2% had persistent proteinuria &gt;0.5 g/day during follow-up.</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated limitations: missing data for several covariates (smoking, BMI, urine occult blood, some Oxford-classification/eGFR/proteinuria measurements) not always recorded at clinic visits; residual confounding by indication ("patients with more severe disease may have been more likely to receive intensive treatment"); hypertension defined by an older (≥140/90) rather than contemporary CKD threshold; "median follow-up duration was approximately 3 years, and the overall occurrence of composite renal events was relatively low," limiting statistical power; regional (single-network) database scope, so out-of-network outcome events may not be captured; unable to distinguish isolated IgAN from IgAN with accompanying renal pathologies. Funded by Otsuka Pharmaceutical Development &amp; Commercialization; no separate conflict-of-interest statement identified beyond this funding disclosure — reviewer-identified potential industry-funding influence to weigh in appraisal. Full text obtained via PMC (PMC13599886).</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr">
+        <is>
+          <t>10.1136/bmjopen-2026-120567 / PMID 42767758 (PMCID PMC13599886)</t>
+        </is>
+      </c>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1136-bmjopen-2026-120567.md (../sources/papers/10.1136-bmjopen-2026-120567.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Hajji et al. 2026 (MCD with mesangial IgA)</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Case Reports in Nephrology</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective clinicopathological case series, n=6 (tier 7 — diagnostic-pitfall carve-out; LOW EVIDENTIARY WEIGHT)</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>6 patients (4 male, 2 female; ages 10–36y at biopsy; onset from early childhood to adulthood), Tunisian referral center, 1995–2025, all presenting with nephrotic syndrome and dominant/exclusive mesangial IgA deposits on immunofluorescence but minimal-change or near-minimal light-microscopy findings (absence of endocapillary proliferation, crescents, necrotizing lesions) — a nosologically contested entity the authors situate "at the interface between MCD and IgAN"</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>None tested (observational clinicopathological description); treatments received: corticosteroids ± cyclophosphamide or mycophenolate mofetil, per case</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>None (single-arm case series; no concurrent classical-proliferative-IgAN comparator group within the paper)</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>All 6 presented with nephrotic-range proteinuria; associated microscopic/macroscopic hematuria and hypertension in some cases. Light microscopy: normal glomeruli (cases 1,2,5) or focal mild mesangial hypercellularity/matrix expansion in 11.5–22% of glomeruli (cases 3,4,6); Oxford M0-E0-S0-T0-C0 or near-minimal profiles predominated (authors note "any Oxford E, S, T, or C lesion favors classical IgAN"). IF: dominant/exclusive mesangial IgA (2–3+) in all cases, with a mesangial "starburst" pattern lacking significant capillary-wall IgA. Electron microscopy unavailable for the entire study period (author-acknowledged limitation). Treatment response: steroid-sensitive/dependent relapsing courses in most cases (60–80% complete-remission rates reported across cases); case 5 sustained remission at 5-year follow-up; case 6 relapsed after MMF discontinuation. Authors propose 3 competing pathogenic hypotheses (incidental IgA trapping; dual glomerulopathy with subclinical IgAN; unified pathogenesis with shared lymphocyte dysregulation) and explicitly do not resolve which applies; they frame correct recognition as important "to avoid diagnostic misclassification and inappropriate therapeutic strategies" versus classical proliferative IgAN, secondary IgA deposits, lupus nephritis, or IgA-dominant postinfectious glomerulonephritis.</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated limitations: electron microscopy unavailable throughout the study period; retrospective design; small case series (n=6) limiting generalizability; no Gd-IgA1 biomarker analysis performed to confirm pathogenic IgA; limited long-term follow-up in some cases. Authors explicitly call for "prospective multicentric studies" with EM and Gd-IgA1 biomarkers. No external funding; authors declare no conflicts of interest. Reviewer-identified: population-boundary judgment call — included under research-question.md's tier-7 diagnostic-pitfall carve-out because the biopsy meets the standard immunofluorescence-based criterion for IgAN (dominant mesangial IgA) and the authors themselves regard the entity as genuinely unsettled/plausibly IgAN-spectrum, not a separately-established distinct disease (contrast row-excluded IgA-IRGN case, see Excluded Candidates table, and full reasoning in this record's own Screening reason). Flagged low evidentiary weight per the tier-7 rule; steroid-responsiveness pattern and small n mean findings should not be generalized to typical proliferative IgAN. Full text obtained via PMC (PMC13595400).</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>10.1155/crin/7021133 / PMID 42774827 (PMCID PMC13595400)</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1155-crin-7021133.md (../sources/papers/10.1155-crin-7021133.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Fejes et al. 2026 (IgAV + medium-vessel arteritis)</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>International Journal of Nephrology and Renovascular Disease</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Single-patient case report (tier 7 — diagnostic-pitfall carve-out; LOW EVIDENTIARY WEIGHT)</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>1 patient, 70-year-old Caucasian male, no significant prior comorbidities; presented with persistent hiccups, generalized weakness, intermittent fever, bilateral thigh pain/myalgia, and later lower-extremity purpura</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>None tested (diagnostic/pathological case description); treatment given: oral methylprednisolone 32 mg/day followed by intravenous cyclophosphamide (cumulative 3900 mg)</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>None (single case; no comparator)</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Markedly elevated CRP (peak 313 mg/L) and procalcitonin (peak 1.29 ng/mL); non-nephrotic proteinuria (PCR 83.7 mg/mmol) with microscopic hematuria; ANCA/ANA/myositis-antibody-negative; infectious workup negative. Kidney biopsy: IgA glomerulonephritis (Oxford M0 E0 S0 T0 C1; diffuse-global granular mesangial IgA 3+ with kappa/lambda, faint IgM/C3) interpreted, in the context of purpura, as a manifestation of IgA vasculitis; concurrently, 3 arcuate arteries showed sclerosing-phase necrotizing arteritis (disrupted internal elastic lamina, tunica-media fibrosis, no active fibrinoid necrosis/inflammatory infiltrate) — a chronic medium-vessel arterial injury pattern compatible with (but not entirely specific for) healed polyarteritis-nodosa-pattern vasculitis. Authors present 4 competing clinicopathological interpretations (IgAV with atypical medium-vessel extension; polyangiitis-overlap syndrome with two independent processes; PAN-pattern arterial disease with coincidental IgA nephropathy; a shared infection-triggered inflammatory trigger) and do not resolve among them, concluding the evidence "establishes the coexistence... but does not establish their hierarchy, causal relationship, or precise nosological classification." Treatment produced rapid normalization of inflammatory markers and complete clinical remission of active nephritic syndrome, with residual chronic kidney disease persisting without active inflammation at follow-up.</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated limitations: proteinuria/hematuria preceded corticosteroid therapy and purpura onset, suggesting IgA-mediated kidney disease may have developed first (complicating causal sequencing); no skin biopsy/direct immunofluorescence performed, so cutaneous IgAV was never histologically confirmed; kidney biopsy captured only chronic (not active) arterial changes; chronic arterial findings are "not entirely specific for" healed PAN-pattern vasculitis; no angiography for visceral microaneurysms; IgA-dominant glomerulonephritis "cannot be distinguished histologically from IgA nephropathy"; mild Oxford-classification glomerular lesions do not fully explain the systemic inflammatory burden. Funding: University of Szeged Open Access Fund (Grant 8787). Conflicts: one author (L. Kovács) reports consulting fees/honoraria/travel support from AstraZeneca, Roche, CSL Behring, Otsuka, Novartis, AbbVie — reviewer-identified potential industry-relationship disclosure, though not directly tied to a therapy evaluated in this case; other authors declared no competing interests. Reviewer-identified: single case, n=1 — no statistical inference possible; included solely as an illustrative diagnostic/pathological-classification data point, thematically adjacent to (adds to, does not duplicate) the larger IgAV/necrotizing-arteritis case series at row 37 (Ribereau-Gayon et al.) — must not be weighted as independent confirmatory evidence. Full text obtained via PMC (PMC13599793).</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>10.2147/IJNRD.S631443 / PMID 42781540 (PMCID PMC13599793)</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.2147-IJNRD.S631443.md (../sources/papers/10.2147-IJNRD.S631443.md)</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4098,6 +4346,28 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Abu Zaher et al. 2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Excluded on population-definition grounds (research-question.md: patients must have "biopsy-confirmed or clinically diagnosed IgA nephropathy [IgAN], and/or IgA vasculitis") combined with the exclusion criterion "Single-patient case reports that do not illustrate a novel/emerging intervention or diagnostic pitfall [in IgAN/IgAV itself]." Per PubMed's own abstract, the case's central differential — advanced IgAN with an infection-triggered flare versus IgA-dominant infection-related glomerulonephritis (IgA-IRGN) — was left explicitly UNRESOLVED (immunosuppression was withheld because of this uncertainty, and kidney function never recovered), so the paper never establishes a confirmed IgAN diagnosis. IgA-IRGN is treated as a recognized, mechanistically/clinically distinct entity from primary IgAN (see the 2026-09-25 batch-5 header note and this record's own Screening reason for the full resolved consistency rule, applied identically to the analogous Batch 4 Nishiyama et al. case, PMID 42752782, which was never filed as a source record and requires no separate correction).</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1136-bcr-2026-275354.md (../sources/papers/10.1136-bcr-2026-275354.md)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 58-67 + background)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4037,6 +4037,626 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Audemard-Verger et al. 2026 (EULAR-style adult IgAV guideline)</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Nature Reviews Rheumatology</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>European multidisciplinary evidence-based practice guideline, systematic-review-informed expert consensus (evidence-synthesis tier placed alongside tier 1 — see judgment call #2 precedent, rows 4–5)</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Adults with IgA vasculitis (IgAV) — international scope, 31-author European multidisciplinary panel (nephrology/rheumatology/dermatology/vasculitis experts)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>None tested directly — guideline provides 14 recommendation statements plus overarching principles for diagnosis, assessment, treatment, and follow-up of adult-onset IgAV, developed via systematic literature review and expert consensus</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable (guideline)</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Per abstract (full text not obtained this batch — see Quality notes): guideline addresses the absence of validated adult-onset IgAV diagnostic criteria and IgAV-specific standardized disease-activity scores; identifies GI complications as the main determinant of short-term outcomes and kidney involvement/CKD-progression risk as the major determinant of long-term prognosis; states that "the treatment of adult-onset IgAV is limited by the paucity of high-quality clinical trials and standardized therapeutic approaches." The specific content of the 14 recommendation statements (e.g., which drugs/thresholds/algorithms are recommended) is NOT extractable from the available text — abstract-level extraction only; full guideline text was not obtained this batch.</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Consensus/systematic-review-informed guideline, not new primary data — recommendations synthesize existing trial evidence already captured elsewhere in this table (rows 1, 37–43, 46, etc.), not independent confirmation. Large 31-author multidisciplinary European panel is a methodological strength; shares co-authors (Barratt, Jayne, Floege, Trivioli) with other studies/guidelines already on file, as previously noted for the Vivarelli et al. IPNA guideline (rows 4–5). Reviewer-identified: full text not obtained this batch (Nature Reviews Rheumatology is subscription-access; not attempted given bounded incremental scope) — `research-writer` must treat the specific recommendation content as unverified pending full-text review, and should not describe individual numbered recommendations beyond what is stated here. The abstract's own acknowledgment of a "paucity of high-quality clinical trials" in adult IgAV is consistent with (not conflicting with) the sparse/null evidence base already documented at rows 1 (Cochrane) and 38 (Rohner et al.). Fills a notable adult-specific guideline gap complementing the pediatric-only Vivarelli et al. 2024 IPNA guideline (rows 4–5) — this is IgAV-specific, not an IgAN extrapolation.</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr">
+        <is>
+          <t>10.1038/s41584-026-01420-3 / PMID 42625065</t>
+        </is>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1038-s41584-026-01420-3.md (../sources/papers/10.1038-s41584-026-01420-3.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Novak et al. 2025 — IgAN</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Kidney International</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Mechanistic immunopathology study, human kidney-biopsy confocal microscopy with correlation to MEST-C (tier 6)</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>17 patients with biopsy-proven IgAN (native-kidney biopsies, Cedars-Sinai Medical Center, Los Angeles, 2012–2019); plus 3 additional IgAN patients' pooled archived biopsies used solely for C3 immunoblot confirmation</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>None (observational) — multi-fluorochrome staining and high-resolution confocal microscopy for glomerular C3, IgA, and IgG pairwise colocalization (Pearson correlation coefficient)</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>None (descriptive; colocalization data correlated against Oxford MEST-C scores within the same cohort)</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>All 17 IgAN biopsies showed C3, IgA, and IgG staining, including biopsies previously read as C3- or IgG-negative by routine immunofluorescence. C3-IgA colocalization was significantly greater than C3-IgG or IgA-IgG (p&lt;0.0001 for each); C3-IgG vs. IgA-IgG did not differ (p=0.0603). C3-IgA colocalization was significantly greater in biopsies with mesangial hypercellularity M1 (p=0.047), endocapillary hypercellularity E1 (p=0.018), and cellular/fibrocellular crescents C1+2 (p=0.019) vs. M0/E0/C0; mean Pearson r was &gt;0.7 (strong colocalization) for all biopsies with any M, E, S, or C lesion present. No difference by S or T score. A mixed-model analysis found a significant positive correlation between the sum of M+E+C scores and C3-IgA colocalization. SDS-PAGE immunoblotting of extracted immune-complex deposits (3 additional patients) confirmed α and β chains of intact complement C3 (not C3b/iC3b) within the deposits.</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>UNRESOLVED CORRIGENDUM CAVEAT (see judgment call #9): a corrigendum/erratum exists for this article (PMID 42760012, DOI 10.1016/j.kint.2026.06.005, "Published Erratum") whose substantive content could not be accessed by `literature-scout` through PubMed or Crossref (existence/linkage confirmed only). Handled identically to the Maisons et al. 2026 precedent (row 40): RETAINED as Included (tier 6), but the Pearson-r/p-values above have NOT been checked against the corrigendum's correction — `research-writer` must state this caveat wherever these specific numbers are cited. Author-stated limitations: no clinical/laboratory follow-up data to link colocalization findings to kidney outcomes; no contemporaneous serum samples to compare circulating vs. deposited immune-complex composition. Reviewer-identified: single-center (Cedars-Sinai), small n=17, retrospective archived-frozen-tissue selection (storage/handling-artifact risk); cross-sectional/correlational design cannot itself establish causality (though the paper cites supporting passive-transfer mouse data). Cross-reference rows 3 (Ștefan et al., MEST-C/complement systematic review) and 39 (Barbour et al., MEST-C/IgAVN outcome cohort) — converges with and mechanistically extends the complement-pathway/active-lesion association, supporting the biological rationale for complement-targeted therapies (rows 16–19, 27–28).</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.kint.2025.07.038 / PMID 40992572 (PMCID PMC12626161)</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.kint.2025.07.038.md (../sources/papers/10.1016-j.kint.2025.07.038.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Novak et al. 2025 — IgAVN</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Kidney International</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Mechanistic immunopathology study, human kidney-biopsy confocal microscopy with correlation to MEST-C (tier 6)</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>23 patients with biopsy-proven IgA vasculitis nephritis (17 pediatric + 6 adult, combined per author-stated sample-size constraint), biopsies from multiple outside hospitals processed/interpreted at Cedars-Sinai, 2010–2019</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>None (observational) — same multi-fluorochrome confocal colocalization method as row 59</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>None (descriptive within-cohort correlation against MEST-C/ISKDC; also compared against the row-59 IgAN cohort for a cross-disease contrast)</t>
+        </is>
+      </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>All 23 IgAVN biopsies showed C3, IgA, and IgG staining, including previously IF-negative cases. C3-IgA colocalization was significantly greater than C3-IgG (p=0.0001); C3-IgA vs. IgA-IgG and IgA-IgG vs. C3-IgG did not differ (p=0.1175, p=0.1003). Cross-disease comparison vs. IgAN (row 59): C3-IgA colocalization was similarly high in both diseases (0.712 IgAN vs. 0.658 IgAVN, p=0.142 — not significantly different); C3-IgG and IgA-IgG colocalization were significantly HIGHER in IgAVN than IgAN (C3-IgG: 0.504 vs. 0.362, p&lt;0.001; IgA-IgG: 0.585 vs. 0.468, p=0.001), and IgAVN biopsies showed more prominent peripheral glomerular capillary-wall deposits than IgAN's predominantly mesangial pattern — a disease-discriminating finding. Unlike IgAN, individual MEST-C components showed only non-significant trends toward higher C3-IgA colocalization in IgAVN (E1 0.678 vs. E0 0.564, p=0.090; C1+2 0.698 vs. C0 0.607, p=0.079), though the sum M+E+C score reached significance for C3-IgA (as in IgAN) and, uniquely in IgAVN, also for C3-IgG. Exploratory: biopsies with diffuse (&gt;50% glomeruli) endocapillary hypercellularity had higher C3-IgA colocalization (≥0.715) than focal-E1 or E0 biopsies; biopsies with ≥10% crescents had higher C3-IgA colocalization (0.750±0.070) than &lt;10% (0.617±0.090) or no crescents (0.607±0.108), p=0.010 for the extreme-group comparison.</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>UNRESOLVED CORRIGENDUM CAVEAT — same as row 59 (see judgment call #9); applies equally to this row's numbers (same publication). Author-stated limitation specific to this row: the IgAVN cohort combines 17 pediatric and 6 adult patients due to sample-size constraints — a population-heterogeneity limitation not applicable to the IgAN row. Reviewer-identified: small n=23 (adult subset only n=6) limits power, especially for the exploratory diffuse-vs-focal-E1 and crescent-percentage subgroup analyses; retrospective archived-tissue selection as in row 59. Cross-reference row 39 (Barbour et al.) — that study's clinical finding that E1 (endocapillary hypercellularity) is the key MEST-C predictor of outcome specifically in IgAVN is mechanistically consistent with (though not independently confirmed by) this study's non-significant E1-colocalization trend; the higher C3-IgG/IgA-IgG colocalization and peripheral-capillary deposit pattern in IgAVN vs. IgAN is a notable pathogenic distinction for `research-writer` to represent between the two diseases, per the topic-specific split-reporting constraint.</t>
+        </is>
+      </c>
+      <c r="K61" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.kint.2025.07.038 / PMID 40992572 (PMCID PMC12626161)</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.kint.2025.07.038.md (../sources/papers/10.1016-j.kint.2025.07.038.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Gu et al. 2026 (telitacicept real-world)</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>International Urology and Nephrology</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Single-center, retrospective, self-controlled before-after case series, n=12 (tier 5 — no comparator arm, consistent with the Pei et al. 2026 finerenone precedent, row 35)</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>12 patients with primary IgAN on stable background ACEI/ARB + SGLT2i therapy, China</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Telitacicept (dual BAFF/APRIL inhibitor), add-on for 6 months</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>None (self-controlled; intra-individual baseline-vs-follow-up comparison)</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>24-hour urinary protein decreased significantly at 3 months (p=0.016) and 6 months (p=0.004): median 1.13 g/24h (IQR 0.62–2.24) at baseline → 0.52 g/24h (IQR 0.26–1.33) at 3 months → 0.51 g/24h (IQR 0.15–1.07) at 6 months; clinical remission rate 75.0%. Median eGFR increased from 61.09 to 77.44 mL/min/1.73m² at 6 months (p=0.008); 83.3% of patients showed renal-function improvement. Median urinary RBC count decreased from 159.00 to 15.00 cells/μL (p=0.005); 70.0% of patients with baseline hematuria achieved hematuria remission. Non-HDL-cholesterol decreased significantly (p=0.028); other cardiovascular risk markers remained stable. Adverse events: low incidence (4 cases), all mild.</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>Very small sample (n=12), single-center, retrospective, no placebo/active-comparator arm or untreated control period (self-controlled before-after design only) — cannot rule out regression-to-mean or background-therapy co-effects as alternative explanations. Short follow-up (6 months). Reviewer-identified: real-world/uncontrolled complement to the already-recorded Lv et al. 2022 RCT (row 23, telitacicept vs. placebo) — directionally consistent with that trial's positive signal but not independent confirmatory evidence given the lack of a control group; should not be weighted equivalently to the RCT. No conflict-of-interest/funding statement extractable from the available abstract text.</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s11255-026-05103-6 / PMID 41870741</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s11255-026-05103-6.md (../sources/papers/10.1007-s11255-026-05103-6.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Hölscher et al. 2026 (pathomics/VALIGA)</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Kidney International Reports</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Multicenter retrospective cohort, prognostic digital-pathology model-comparison study (tier 6, diagnostic-technology reading of the mechanistic/novel-target tier — see judgment call #12)</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>555 adults with biopsy-proven IgAN, multicenter European VALIGA cohort, centralized MEST-C histopathology; median age 37.9y, 72% male, 97% White; median follow-up 7.3 years</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>Deep-learning-derived "pathomics" quantitative morphological biomarkers (25 candidate features reduced to 10 via clustering) extracted from digitized PAS-stained whole-slide images</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Traditional Oxford MEST-C histopathology scoring and the existing International IgAN Prediction Tool (IIgAN-PT), both fit in the same cohort for head-to-head comparison</t>
+        </is>
+      </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Primary composite outcome (kidney failure or ≥50% eGFR decline) occurred in 148/555 (27%); 7-year risk 20.2% (95% CI 16.4–23.9), 10-year risk 29.8% (95% CI 24.8–34.5). Pathomics alone (no clinical variables) slightly outperformed MEST-C alone (Δ C-statistic +0.04, 95% CI 0.03–0.06), but was marginally WORSE than MEST-C once clinical predictors (as in IIgAN-PT) were added (Δ C-statistic −0.034, 95% CI −0.042 to −0.027). Adding pathomics on top of the existing IIgAN-PT gave only minor improvement (Δ C-statistic +0.024, 95% CI 0.019–0.028, model without ethnicity); calibration was better without ethnicity adjustment but worse with it. Patient risk-group stratification (4 groups) was consistent between pathomics- and MEST-C-based models. Authors conclude pathomics is "noninferior" to MEST-C — an objective, reproducible alternative rather than a large incremental predictive gain.</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: findings primarily generalizable to European/White populations (97% White); no external validation in an independent cohort (internal bootstrap validation only); retrospective design limits real-world clinical-impact assessment; interaction terms between pathomics and clinical variables not tested due to sample-size constraints. Reviewer-identified: despite the large multicenter sample and centralized histopathology (reducing interobserver variability vs. real-world practice), the incremental predictive gains are small and of uncertain clinical significance — fundamentally a proof-of-concept model-comparison study, not a clinical-outcomes intervention trial. Thematically parallel to Jaugey et al. 2023 (row 32); Hölscher's larger, multicenter, outcome-validated design is comparatively more rigorous within this sub-topic. Two authors disclosed consulting/research-funding relationships with multiple pharmaceutical/AI companies (CSL Vifor, Otsuka, Novartis, Bristol Myers Squibb, Roche, Novo Nordisk, Astellas, aetherAI, BioCryst), stated by the authors as "none relevant to this work" — noted for completeness.</t>
+        </is>
+      </c>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.ekir.2026.106708 / PMID 42661948 (PMCID PMC13519253)</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.ekir.2026.106708.md (../sources/papers/10.1016-j.ekir.2026.106708.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Sun et al. 2026 (Nefecon, Asian-American real-world)</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Clinical Nephrology</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Single-center, retrospective, real-world observational case series with internal exposure-duration subgroup comparison (tier 5)</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>45 consecutive Asian-American adults with IgAN (97.8% Asian), Chinatown Kidney Care practice, New York, USA; mean age at Nefecon initiation 48.1y (SD 13.6); mean follow-up 14.9 months</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Delayed-release budesonide (Nefecon/Tarpeyo), 16 mg/day; background therapies included ARB (87%), mycophenolate mofetil (53%), systemic corticosteroids (29%), SGLT2 inhibitors (22%); 18% also received sparsentan after starting Nefecon</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Internal subgroup comparison: patients completing ≥9 months of Nefecon (n=30, the US-labeled recommended duration) vs. those treated &lt;9 months (n=15); no placebo/untreated comparator</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Overall: eGFR stable at 9 months (mean change +0.9 mL/min/1.73m², SD 10.3); UPCR decreased 19% on average. ≥9-month subgroup: eGFR +3.6 mL/min/1.73m² (SD 10.6), UPCR −26%. &lt;9-month subgroup: eGFR −3.5 mL/min/1.73m² (SD 8.3), UPCR only −3.3%. Over full follow-up: 1 patient (2.2%) reached kidney failure; 30% eGFR reduction in 13% overall (7% in ≥9mo vs. 27% in &lt;9mo); 40% reduction in 7% (3% vs. 13%); 50% reduction in 4% (3% vs. 7%). Adverse events in 16% (7/45), all mild (6) or moderate (1), none severe; 5 patients (11%) permanently discontinued due to AEs (edema/swelling in 4, BP increase in 1) — comparable to NefIgArd's 9% AE-discontinuation rate. Authors explicitly caution that the duration-subgroup comparison reflects differential treatment persistence/confounding by indication (younger, better-baseline-eGFR patients more likely to complete the full course), not a randomized exposure contrast, and "cannot be taken as evidence that longer treatment duration per se causes better outcomes."</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: small, single-center, observational, no comparator/control group; substantial heterogeneity in concurrent background IgAN therapies complicates attribution of outcomes specifically to Nefecon; mean follow-up (~15 months) too short for long-term kidney-failure outcomes. MAJOR COI/FUNDING DISCLOSURE (author-confirmed): study funded by Calliditas Therapeutics (Nefecon's manufacturer, now part of Asahi Kasei Corporation); several authors were Calliditas employees during the study (2 of 9) or received direct funding from Calliditas for study design/conduct/analysis/reporting/medical-writing support (remaining authors) — a materially higher industry-entanglement level (sponsor-employed co-authors, not just sponsor funding) than typical RCT disclosures elsewhere in this table; weight accordingly. Cross-reference rows 13–14 (NefIgArd RCT) — findings are directionally consistent with, not independent confirmation of, the pivotal trial; this study explicitly frames itself as corroborating NefIgArd in an understudied population (Asian-Americans) and an understudied variable (treatment-duration/adherence effects).</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>10.5414/CN112036 / PMID 42596753 (PMCID PMC13621273)</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.5414-CN112036.md (../sources/papers/10.5414-CN112036.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Chen et al. 2026 (TRIM21/AID class-switching)</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>International Immunopharmacology</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>Mixed human PBMC + murine knockout mechanistic study (tier 6)</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Human PBMCs from IgAN patients (exact n not extractable from available abstract text); Trim21-knockout mice subjected to oral mucosal immunization (HSP/IgAN-type model)</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>None as a tested intervention — TRIM21 genetic deletion (mouse) and endogenous TRIM21 expression level (human, observational exposure)</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Implied wild-type mice; human IgAN patients vs. an unspecified comparison group (not detailed in the available abstract)</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>TRIM21 expression was significantly reduced in PBMCs from IgAN patients and inversely correlated with serum IgA levels (exact correlation/p-values not extractable from available text). In Trim21-knockout mice with oral mucosal immunization, TRIM21 deficiency exacerbated the disease phenotype: increased urinary protein-to-creatinine ratio and serum creatinine, impaired intestinal barrier integrity, and expanded IgA⁺ B cells in gut-associated lymphoid tissue. Mechanistically, TRIM21 was proposed to directly bind IκBα and promote its ubiquitination, restraining NF-κB activation and downstream AID (activation-induced cytidine deaminase) expression; TRIM21 loss relieved this suppression, enhancing IgA class switching. Authors conclude a TRIM21-IκBα-NF-κB-AID axis negatively regulates intestinal IgA biosynthesis and propose it as a potential therapeutic target in IgAN.</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>Not extractable from available text: exact sample sizes (human PBMC cohort and mouse groups), specific correlation coefficients/p-values beyond directional significance, and the authors' own stated limitations — full text was not obtained this batch (no PMCID on record), so extraction is abstract/metadata-level only. Reviewer-identified: preclinical/mechanistic only — no clinical efficacy or therapeutic intervention tested in humans; single-center (Central South University, China); the "potential therapeutic target" framing is hypothesis-generating, not yet validated with a targeted intervention. Cross-reference rows 29–30 (Zachova/Zhu, gut-kidney axis) and row 50 (Mayer-Hain, NETosis/PMN mechanism) — extends the mucosal-immunity sub-topic with a novel specific molecular regulator (TRIM21) of the AID-dependent IgA class-switching step not previously captured in this evidence base.</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.intimp.2026.117087 / PMID 42385642</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.intimp.2026.117087.md (../sources/papers/10.1016-j.intimp.2026.117087.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Tanaka et al. 2026 (anti-GBM misattributed to IgAV)</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Pediatric Nephrology</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Single-patient case report (tier 7 — diagnostic-pitfall carve-out)</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>8-year-old girl, pediatric IgA vasculitis nephritis follow-up, Japan</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>None tested — diagnostic recognition case; plasma exchange + immunosuppressive therapy administered once anti-GBM disease was recognized</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>None (single patient)</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Patient developed anti-GBM nephritis initially misattributed to IgAV kidney involvement; diagnosis confirmed by markedly elevated anti-GBM antibodies and kidney-biopsy findings distinct from IgAVN. Despite plasma exchange and immunosuppressive therapy, kidney function deteriorated to kidney failure within several months. Authors' explicit teaching point: "worsening urinary findings or kidney function during follow-up of IgAV should prompt consideration of RPGN and appropriate serological screening, as well as timely kidney biopsy, rather than being attributed solely to IgAV nephritis."</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>N=1 — no statistical inference possible; included solely as an illustrative diagnostic-pitfall example per the tier-7 carve-out, not as efficacy or epidemiological evidence. Author-stated: early recognition of anti-GBM disease is essential, as delayed diagnosis leads to irreversible kidney damage — this case itself illustrates a diagnostic delay with a poor outcome (progression to kidney failure) despite treatment once recognized. Reviewer-identified: fits the tier-7 "clinically significant diagnostic pitfall" criterion more unambiguously than several other borderline case reports in this evidence base (e.g., rows 66–67 below), given the paper's own explicit framing as "a diagnostic challenge" with a clear, generalizable clinical teaching point (a competing alternate primary diagnosis, directly analogous to rows 56–57's diagnostic-pitfall cases).</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s00467-026-07337-z / PMID 42084625 (PMCID PMC13481406)</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s00467-026-07337-z.md (../sources/papers/10.1007-s00467-026-07337-z.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Suleman et al. 2026 (fatal adult IgAV, GI + possible cardiac)</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Cureus</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Single-patient case report (tier 7 — diagnostic-pitfall carve-out; BORDERLINE judgment call, see judgment call #10; LOW EVIDENTIARY WEIGHT)</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>50-year-old man, biopsy-proven IgA nephropathy, pre-existing seropositive rheumatoid arthritis, type 2 diabetes, hypertension, heart failure with reduced ejection fraction (dilated cardiomyopathy); developed clinically diagnosed (not biopsy-confirmed) adult-onset IgA vasculitis with purpura, polyarthralgia, GI involvement (bloody stools, CT-confirmed small-bowel inflammation, ileus) and apparent renal flare, plus a fatal cardiac event of uncertain causal relationship to the vasculitis; United Kingdom</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Escalating corticosteroids (oral then IV hydrocortisone) followed by rituximab 1000mg IV (single dose) for corticosteroid-refractory multisystem disease</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>None (single patient, pre/post within-case)</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Initial clinical/biochemical improvement (GI symptoms, renal function) within one week of rituximab; patient discharged with a planned corticosteroid taper and a second rituximab dose scheduled. One day after discharge, re-presented with STEMI (troponin 1705 ng/L, proximal LAD occlusion) treated with PCI/stenting; subsequently suffered a ventricular fibrillation (VF) arrest, was resuscitated, then developed GI bleeding (endoscopy showed only moderate duodenitis, "insufficient to explain" the bleeding severity) and a second, fatal VF arrest despite a patent LAD stent on repeat angiography (no new obstructive lesion). The paper extensively discusses — but cannot resolve — whether the cardiac events reflect vasculitic/inflammatory coronary or microvascular involvement versus the patient's substantial pre-existing cardiovascular disease; no coronary or myocardial histopathology was obtained. Explicit authors' learning point: "Cardiac complications occurring during IgA vasculitis require careful differential assessment, particularly in patients with pre-existing cardiovascular disease."</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>N=1, fatal outcome — no statistical inference possible. Author-stated (explicit "Diagnostic limitations" section): absence of contemporaneous histopathological confirmation of the cutaneous/GI manifestations (clinically attributed only, not biopsied); no cardiac biomarker, serological marker, angiographic feature, or tissue biopsy specifically demonstrated coronary vasculitis — cardiac events are "presented as possibly associated with IgA vasculitis rather than definitively caused by it." BORDERLINE JUDGMENT CALL (see judgment call #10): included under the tier-7 diagnostic-pitfall prong on a LOWER-CONFIDENCE basis than row 65 — this is a causal-attribution pitfall for a complication, not a competing-alternate-diagnosis pitfall. Rituximab itself is not a novel/emerging intervention in this evidence base (already represented at rows 26, 46) and its use here does not independently support inclusion. `Research-writer` must not extrapolate a generalizable "cardiac involvement in IgAV" epidemiological claim from this single, multiply-confounded, fatal case. No conflict-of-interest/funding statement extractable from the available full text.</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>10.7759/cureus.116913 / PMID 42799210 (PMCID PMC13614159)</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.7759-cureus.116913.md (../sources/papers/10.7759-cureus.116913.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Watanabe et al. 2026 (T-DM1-induced IgAV)</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Internal Medicine (Tokyo)</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Single-patient case report (tier 7 — novel/emerging-mechanism carve-out; BORDERLINE judgment call, see judgment call #11; LOW EVIDENTIARY WEIGHT)</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Elderly woman undergoing trastuzumab emtansine (T-DM1) therapy for HER2-positive breast cancer, Japan</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>T-DM1 (ado-trastuzumab emtansine, anti-HER2 antibody-drug conjugate) as the causative/triggering agent (not a therapeutic intervention for IgAV); subsequently treated with prednisolone + cyclophosphamide for the resulting IgAV</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>None (single patient)</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Patient presented with purpura, hematuria, proteinuria, and decreased renal function during T-DM1 treatment. Skin biopsy confirmed leukocytoclastic vasculitis with IgA deposition (biopsy-confirmed IgAV diagnosis). Treatment with prednisolone + cyclophosphamide achieved clinical remission. A follow-up renal biopsy at 5 months post-treatment showed persistent mild proliferative glomerulonephritis with fibrotic crescent formation despite clinical remission — i.e., ongoing subclinical histologic activity. Authors conclude this represents T-DM1-associated (drug-induced) IgA vasculitis and emphasize "awareness of the possibility of serious adverse effects associated with drug administration."</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>N=1 — no statistical/causal inference possible beyond temporal association; no formal pharmacovigilance causality-assessment instrument (e.g., Naranjo score) reported in the available abstract. BORDERLINE JUDGMENT CALL (see judgment call #11): included under the tier-7 "novel/emerging mechanism" prong — a newly recognized drug-induced pathogenic trigger for IgAV, relevant to research-question.md's "pathogenic mechanisms or pathways" scope and to oncology/nephrology pharmacovigilance. This is a LOWER-CONFIDENCE fit than row 65 and must not be read as establishing T-DM1 as a confirmed, generalizable IgAV risk factor from a single case. No conflict-of-interest/funding statement extractable from the available abstract.</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>10.2169/internalmedicine.6751-25 / PMID 41780977</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.2169-internalmedicine.6751-25.md (../sources/papers/10.2169-internalmedicine.6751-25.md)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4048,7 +4668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4279,6 +4899,80 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.1007-s10067-023-06781-8.md (../sources/papers/10.1007-s10067-023-06781-8.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Wade et al. 2026</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Pediatric Nephrology</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Complement biology and complement-targeted therapeutics across glomerular diseases, using IgAN as the illustrative worked example</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Include – background/context only (tier 8 narrative review per research-question.md's study-type ladder: "narrative reviews — usable for background/context only, never as a primary evidence source"). No original data. May be used for framing/orientation on complement-targeted-therapy rationale; must not be cited as the evidentiary basis for any specific quantitative or study-level claim — see rows 3, 16–19, 27–28, 47, 49, 59–60 for the primary complement-pathway evidence.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s00467-026-07166-0 / PMID 41714421</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s00467-026-07166-0.md (../sources/papers/10.1007-s00467-026-07166-0.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Filippatos et al. 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Rheumatology International</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Infectious triggers and immunopathogenic mechanisms in pediatric IgA vasculitis</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Include – background/context only (tier 8 narrative review per research-question.md's study-type ladder). Authors explicitly disclaim systematic-review/PRISMA completeness ("no systematic-review or PRISMA completeness claim is made") despite an underlying structured PubMed/MEDLINE search, and report no original primary data of their own. May be used for background/orientation on infectious-trigger epidemiology (group A streptococcus and seasonal respiratory bacteria most consistently associated; lower-certainty case-based evidence for Mycoplasma pneumoniae/H. pylori/SARS-CoV-2/enteric-parasitic triggers; no consistent excess risk from vaccination); must not be cited as the evidentiary basis for a specific quantitative claim.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>10.1007/s00296-026-06295-x / PMID 42799772</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s00296-026-06295-x.md (../sources/papers/10.1007-s00296-026-06295-x.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 68-70)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4654,6 +4654,192 @@
       <c r="L68" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.2169-internalmedicine.6751-25.md (../sources/papers/10.2169-internalmedicine.6751-25.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Lin et al. 2026</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Renal Failure</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Single-center retrospective cohort study (tier 4)</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>180 patients with biopsy-proven IgAN and ≥3 years of clinical follow-up; China (Zhongshan Hospital [Xiamen], Fudan University)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>Baseline/longitudinal clinical and histopathologic factors (ln[UACR+1] [albuminuria], Oxford MEST-C "T" lesion category [T0/T1/T2]) analyzed as predictors of eGFR trajectory — no therapeutic intervention tested</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>None (single-cohort observational; internal comparison of T1/T2 vs. T0 as reference within the multivariable model)</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Median eGFR slope −1.12 mL/min/1.73m²/year; 35/180 (19.4%) met the operational rapid-progression threshold (&lt;−5 mL/min/1.73m²/year). In the primary multivariable model: higher ln(UACR+1) predicted steeper decline (β=−0.612, 95% CI −1.073 to −0.150); Oxford T2 lesions predicted 3.87 mL/min/1.73m²/year faster loss vs. T0 (β=−3.870, 95% CI −7.087 to −0.654); T1 did not differ from T0. Model R²=0.159 (adjusted R²=0.130). UACR and T2 point estimates remained negative under HC3 robust inference and after excluding influential observations, but the T2 association was less stable in some restricted analyses.</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated: baseline albuminuria was the most consistent adverse marker of eGFR slope; the T2-lesion association, while directionally consistent, derived from only 16/180 patients (8.9%) and lost statistical significance when the analysis was restricted to patients with ≥5 eGFR measurements — authors explicitly characterize this as "tentative" and "strictly hypothesis-generating," not a confirmed finding. Reviewer-identified: single-center, retrospective design with no treatment comparator; modest model fit (R²=0.159) leaves most eGFR-slope variance unexplained; ≥3-year-follow-up inclusion requirement may introduce survivorship/selection bias against rapidly progressing or lost-to-follow-up patients; single Chinese-population center limits generalizability.</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>10.1080/0886022X.2026.2732704 / PMID 42844235</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1080-0886022X.2026.2732704.md (../sources/papers/10.1080-0886022X.2026.2732704.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Chen et al. 2026 (renal-tissue/PBMC secretory-protein &amp; crotonylomics)</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Journal of Proteomics</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Exploratory human-sample multi-omics mechanistic study, unpaired cross-sectional cohorts (tier 6)</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>48 samples total: renal tissue from 7 IgAN patients vs. 10 controls; PBMCs from 6 IgAN patients vs. 25 controls; China</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>None tested — observational proteomic (renal tissue) and crotonylation/Kcr (PBMC) profiling comparing IgAN patients to non-IgAN controls, with PPI network analysis, functional enrichment, transcription-factor prediction, and DSigDB/Enrichr compound-enrichment analysis</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>IgAN patients vs. non-IgAN controls (separate renal-tissue and PBMC cohorts; not paired within individuals)</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>92 differentially abundant HPA-annotated secretory proteins identified in IgAN renal tissue vs. controls; 36 secretory proteins with differential protein-abundance-normalized Kcr signals (120 Kcr sites) in IgAN PBMCs vs. controls. PPI network analysis prioritized 10 exploratory hub candidates (FGA, FGB, A2M, APOA1, C3, HP, SERPINA1, APOB, FGG, TF/transferrin). STAT1, PML, STAT5B, and MYH11 were computationally predicted as candidate upstream transcription factors. DSigDB/Enrichr compound-enrichment analysis flagged thapsigargin as a database-derived, hypothesis-generating compound associated with the secretory-protein network.</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated (quoted): "Because the datasets were unpaired and the proteomic and crotonylomic samples were pooled within groups, the results do not establish participant-level cross-tissue relationships, causal regulation, validated biomarkers, or therapeutic efficacy. Larger individual-level cohorts and functional studies are required for validation." Authors explicitly frame the study as providing only "exploratory molecular insights" despite the limited sample size. Reviewer-identified: very small group sizes (as few as 6–10 per arm); renal-tissue and PBMC cohorts are not from the same individuals (no cross-tissue correlation possible); single-center/single-country; hub proteins and upstream TFs are computational predictions, not experimentally validated; no clinical/functional validation performed — findings should be treated as hypothesis-generating only, not as established IgAN biomarkers or mechanisms. Cross-reference rows 45/47–49 (other tier-6 mechanistic/multi-omics IgAN studies in this evidence base) for the broader mechanistic-evidence landscape; this study adds a distinct secretory-protein/lysine-crotonylation angle not previously captured.</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>10.1016/j.jprot.2026.105737 / PMID 42843589</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1016-j.jprot.2026.105737.md (../sources/papers/10.1016-j.jprot.2026.105737.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Loudon et al. 2026 (hepatic/GI-guided treatment in adult IgAV)</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>BMJ Case Reports</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>Single-patient case report (tier 7 — novel/emerging management-nuance carve-out; BORDERLINE judgment call, see judgment call #13; LOW EVIDENTIARY WEIGHT)</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Man in his 20s, no prior medical history, biopsy-confirmed IgAV (perivascular IgA deposition on skin, ileal, and renal biopsies); Australia (Cairns Hospital)</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>6-week oral prednisone course, initiated after multidisciplinary consultation, triggered by recurrent severe gastrointestinal symptoms (ileal ulceration on colonoscopy) PLUS biochemical evidence of hepatic involvement — despite renal involvement (subnephrotic-range proteinuria) alone not meeting the authors' stated usual treatment threshold</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>None (single patient, pre/post within-case)</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>Symptoms resolved on the 6-week prednisone course, with complete normalisation of renal function and liver enzymes.</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Author-stated (quoted): "Immunosuppressive treatment is typically reserved for significant renal involvement or refractory abdominal and joint pain. However, therapeutic targets for gastrointestinal involvement remain poorly defined." BORDERLINE JUDGMENT CALL (see judgment call #13): per the authors' own framing, treating refractory GI/joint symptoms is already a standard indication — not itself novel — so the genuinely novel/emerging element supporting tier-7 inclusion is specifically that biochemical hepatic involvement (an uncommon, poorly characterized IgAV manifestation) was an explicit co-trigger for treatment alongside GI symptoms. This is a LOWER-CONFIDENCE, contestable fit, flagged to the orchestrator/user for possible review, consistent with the standard applied to the Suleman et al. 2026 and Watanabe et al. 2026 judgment calls (rows 66–67). Reviewer-identified: N=1, no statistical inference possible; no liver biopsy was performed (biochemical evidence only), so causal attribution of the liver-enzyme derangement specifically to IgAV (vs. an alternative etiology) is not conclusively established in the available text; a single favorable outcome cannot be generalized into a validated treatment indication. No conflict-of-interest/funding statement extractable from the available abstract.</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>10.1136/bcr-2026-275498 / PMID 42833852</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1136-bcr-2026-275498.md (../sources/papers/10.1136-bcr-2026-275498.md)</t>
         </is>
       </c>
     </row>
@@ -4987,7 +5173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5062,6 +5248,28 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Yuji &amp; Yuji 2026</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Excluded per the conservative default under the anti-fabrication rules: bibliographic identity is `verified`, but despite an independent evidence-reviewer re-attempt (WebFetch on the DOI, which 302-redirects to the Springer landing page, which 303-redirects to a Springer authentication/paywall gate; `get_article_metadata` confirms no abstract is on file and the article type is "Letter" only, not "Letter"+"Case Reports"), the full text/abstract remain completely inaccessible, so it cannot be confirmed whether this is a data-bearing research letter (would be a primary-evidence candidate) or a no-original-data commentary (research-question.md's exclusion criterion: "Editorials, letters, or commentaries with no original data [background-context use only, never as an evidence-table entry]"). Not placed in Background/Context either, since that section requires confirming the record meets an inclusion-criteria-satisfying profile (e.g., a genuine tier-8 narrative review), which cannot be confirmed without readable content. Flagged to orchestrator: if institutional/alternative full-text access to this letter becomes available, it should be sent back for re-screening — topically it is a direct, named-drug (telitacicept) IgAN match and would be relevant if it turns out to report original vaccination/humoral-response data.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1007-s11255-026-05421-9.md (../sources/papers/10.1007-s11255-026-05421-9.md)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 71-72)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -54,7 +54,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -424,21 +424,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -561,7 +561,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1002-14651858.CD005128.pub4.md (../sources/papers/10.1002-14651858.CD005128.pub4.md)</t>
+          <t>sources/papers/10.1002-14651858.CD005128.pub4.md</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1371-journal.pone.0323530.md (../sources/papers/10.1371-journal.pone.0323530.md)</t>
+          <t>sources/papers/10.1371-journal.pone.0323530.md</t>
         </is>
       </c>
     </row>
@@ -685,7 +685,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2023.11.005.md (../sources/papers/10.1016-j.ekir.2023.11.005.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2023.11.005.md</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-024-06502-6.md (../sources/papers/10.1007-s00467-024-06502-6.md)</t>
+          <t>sources/papers/10.1007-s00467-024-06502-6.md</t>
         </is>
       </c>
     </row>
@@ -809,7 +809,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-024-06502-6.md (../sources/papers/10.1007-s00467-024-06502-6.md)</t>
+          <t>sources/papers/10.1007-s00467-024-06502-6.md</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-S0140-6736(23)00569-X.md (../sources/papers/10.1016-S0140-6736(23)00569-X.md)</t>
+          <t>sources/papers/10.1016-S0140-6736(23)00569-X.md00569-X.md)</t>
         </is>
       </c>
     </row>
@@ -933,7 +933,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-S0140-6736(23)02302-4.md (../sources/papers/10.1016-S0140-6736(23)02302-4.md)</t>
+          <t>sources/papers/10.1016-S0140-6736(23)02302-4.md02302-4.md)</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.2215-CJN.0000000961.md (../sources/papers/10.2215-CJN.0000000961.md)</t>
+          <t>sources/papers/10.2215-CJN.0000000961.md</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1093-ndt-gfae021.md (../sources/papers/10.1093-ndt-gfae021.md)</t>
+          <t>sources/papers/10.1093-ndt-gfae021.md</t>
         </is>
       </c>
     </row>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-S0140-6736(26)00960-8.md (../sources/papers/10.1016-S0140-6736(26)00960-8.md)</t>
+          <t>sources/papers/10.1016-S0140-6736(26)00960-8.md00960-8.md)</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1681-ASN.0000001076.md (../sources/papers/10.1681-ASN.0000001076.md)</t>
+          <t>sources/papers/10.1681-ASN.0000001076.md</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1681-ASN.0000001097.md (../sources/papers/10.1681-ASN.0000001097.md)</t>
+          <t>sources/papers/10.1681-ASN.0000001097.md</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2022.09.017.md (../sources/papers/10.1016-j.kint.2022.09.017.md)</t>
+          <t>sources/papers/10.1016-j.kint.2022.09.017.md</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-S0140-6736(23)01554-4.md (../sources/papers/10.1016-S0140-6736(23)01554-4.md)</t>
+          <t>sources/papers/10.1016-S0140-6736(23)01554-4.md01554-4.md)</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2023.02.012.md (../sources/papers/10.1016-j.kint.2023.02.012.md)</t>
+          <t>sources/papers/10.1016-j.kint.2023.02.012.md</t>
         </is>
       </c>
     </row>
@@ -1491,7 +1491,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2023.09.027.md (../sources/papers/10.1016-j.kint.2023.09.027.md)</t>
+          <t>sources/papers/10.1016-j.kint.2023.09.027.md</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1056-NEJMoa2410316.md (../sources/papers/10.1056-NEJMoa2410316.md)</t>
+          <t>sources/papers/10.1056-NEJMoa2410316.md</t>
         </is>
       </c>
     </row>
@@ -1615,7 +1615,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1056-NEJMoa2600743.md (../sources/papers/10.1056-NEJMoa2600743.md)</t>
+          <t>sources/papers/10.1056-NEJMoa2600743.md</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2023.01.041.md (../sources/papers/10.1016-j.ekir.2023.01.041.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2023.01.041.md</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1739,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1056-NEJMoa2305635.md (../sources/papers/10.1056-NEJMoa2305635.md)</t>
+          <t>sources/papers/10.1056-NEJMoa2305635.md</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2024.03.012.md (../sources/papers/10.1016-j.kint.2024.03.012.md)</t>
+          <t>sources/papers/10.1016-j.kint.2024.03.012.md</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2022.05.017.md (../sources/papers/10.1016-j.ekir.2022.05.017.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2022.05.017.md</t>
         </is>
       </c>
     </row>
@@ -1925,7 +1925,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2022.12.014.md (../sources/papers/10.1016-j.ekir.2022.12.014.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2022.12.014.md</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-025-06905-z.md (../sources/papers/10.1007-s00467-025-06905-z.md)</t>
+          <t>sources/papers/10.1007-s00467-025-06905-z.md</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-025-06905-z.md (../sources/papers/10.1007-s00467-025-06905-z.md)</t>
+          <t>sources/papers/10.1007-s00467-025-06905-z.md</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.5414-CN111984.md (../sources/papers/10.5414-CN111984.md)</t>
+          <t>sources/papers/10.5414-CN111984.md</t>
         </is>
       </c>
     </row>
@@ -2173,7 +2173,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1681-ASN.0000000534.md (../sources/papers/10.1681-ASN.0000000534.md)</t>
+          <t>sources/papers/10.1681-ASN.0000000534.md</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2235,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.2215-CJN.0000000000000384.md (../sources/papers/10.2215-CJN.0000000000000384.md)</t>
+          <t>sources/papers/10.2215-CJN.0000000000000384.md</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1681-ASN.2021081086.md (../sources/papers/10.1681-ASN.2021081086.md)</t>
+          <t>sources/papers/10.1681-ASN.2021081086.md</t>
         </is>
       </c>
     </row>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1093-ndt-gfae052.md (../sources/papers/10.1093-ndt-gfae052.md)</t>
+          <t>sources/papers/10.1093-ndt-gfae052.md</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2421,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1681-ASN.0000000000000465.md (../sources/papers/10.1681-ASN.0000000000000465.md)</t>
+          <t>sources/papers/10.1681-ASN.0000000000000465.md</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1093-ndt-gfad039.md (../sources/papers/10.1093-ndt-gfad039.md)</t>
+          <t>sources/papers/10.1093-ndt-gfad039.md</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.phymed.2026.158684.md (../sources/papers/10.1016-j.phymed.2026.158684.md)</t>
+          <t>sources/papers/10.1016-j.phymed.2026.158684.md</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.3390-ijms25084383.md (../sources/papers/10.3390-ijms25084383.md)</t>
+          <t>sources/papers/10.3390-ijms25084383.md</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1080-0886022X.2026.2681246.md (../sources/papers/10.1080-0886022X.2026.2681246.md)</t>
+          <t>sources/papers/10.1080-0886022X.2026.2681246.md</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1080-07853890.2026.2720379.md (../sources/papers/10.1080-07853890.2026.2720379.md)</t>
+          <t>sources/papers/10.1080-07853890.2026.2720379.md</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2793,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1080-08916934.2026.2677546.md (../sources/papers/10.1080-08916934.2026.2677546.md)</t>
+          <t>sources/papers/10.1080-08916934.2026.2677546.md</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1093-ndt-gfae009.md (../sources/papers/10.1093-ndt-gfae009.md)</t>
+          <t>sources/papers/10.1093-ndt-gfae009.md</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.2215-CJN.0000000000000398.md (../sources/papers/10.2215-CJN.0000000000000398.md)</t>
+          <t>sources/papers/10.2215-CJN.0000000000000398.md</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>CAVEAT (updated 2026-09-13, following `literature-scout`'s Run 19 follow-up): a published corrigendum (Erratum) exists for this article — PMID 42457434, DOI 10.1016/j.ejim.2026.107059, Eur J Intern Med 151:107059. Its *existence* and formal "Published Erratum" classification (as opposed to a retraction or expression of concern) are now confirmed. Its *substantive content* — what specific figure, cluster definition, or number was corrected — remains inaccessible: an exhaustive 10-step verification attempt (PubMed metadata, PMC lookup, DOI resolution, direct ScienceDirect/PDF fetch [403 Forbidden], Crossref, Unpaywall, EuropePMC, reformulated web searches, and the EFIM reprint page — full detail in `sources/search-log.md` Run 19 and the dated addendum in this study's source-record Verification notes) found every full-text path either paywalled, a bare redirect/metadata stub, or abstract-empty. This upgrades the caveat from "not yet checked" to "actively verified as currently inaccessible despite exhaustive effort" — a materially stronger disclosure, though the underlying uncertainty about whether/how the cluster findings above (n=260/n=208, phenotype definitions) were affected by the correction is unchanged and genuinely unresolved. RETAINED as Included (tier 4), not downgraded or excluded, because (a) the confirmed "Published Erratum" classification typically denotes correction of a discrete error rather than invalidation of the study, and (b) the independent two-country (French/Slovenian) validation of the clustering result is a structural methodological strength unlikely to be nullified by a typical erratum-level correction. `research-writer` must present this row's specific figures with this caveat explicitly stated (not as settled numbers) and must not treat the exhausted verification effort as having resolved the uncertainty — it only rules out further easy resolution; full resolution would require institutional/subscription access to ScienceDirect or direct correspondence with the journal/authors. Otherwise a notable methodological strength: independent two-country validation of the clustering result.</t>
+          <t>CAVEAT (updated 2026-09-13, following `literature-scout`'s Run 19 follow-up): a published corrigendum (Erratum) exists for this article — PMID 42457434, DOI 10.1016/j.ejim.2026.107059, Eur J Intern Med 151:107059. Its existence and formal "Published Erratum" classification (as opposed to a retraction or expression of concern) are now confirmed. Its substantive content — what specific figure, cluster definition, or number was corrected — remains inaccessible: an exhaustive 10-step verification attempt (PubMed metadata, PMC lookup, DOI resolution, direct ScienceDirect/PDF fetch [403 Forbidden], Crossref, Unpaywall, EuropePMC, reformulated web searches, and the EFIM reprint page — full detail in `sources/search-log.md` Run 19 and the dated addendum in this study's source-record Verification notes) found every full-text path either paywalled, a bare redirect/metadata stub, or abstract-empty. This upgrades the caveat from "not yet checked" to "actively verified as currently inaccessible despite exhaustive effort" — a materially stronger disclosure, though the underlying uncertainty about whether/how the cluster findings above (n=260/n=208, phenotype definitions) were affected by the correction is unchanged and genuinely unresolved. RETAINED as Included (tier 4), not downgraded or excluded, because (a) the confirmed "Published Erratum" classification typically denotes correction of a discrete error rather than invalidation of the study, and (b) the independent two-country (French/Slovenian) validation of the clustering result is a structural methodological strength unlikely to be nullified by a typical erratum-level correction. `research-writer` must present this row's specific figures with this caveat explicitly stated (not as settled numbers) and must not treat the exhausted verification effort as having resolved the uncertainty — it only rules out further easy resolution; full resolution would require institutional/subscription access to ScienceDirect or direct correspondence with the journal/authors. Otherwise a notable methodological strength: independent two-country validation of the clustering result.</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ejim.2026.106742.md (../sources/papers/10.1016-j.ejim.2026.106742.md)</t>
+          <t>sources/papers/10.1016-j.ejim.2026.106742.md</t>
         </is>
       </c>
     </row>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1097-MD.0000000000036521.md (../sources/papers/10.1097-MD.0000000000036521.md)</t>
+          <t>sources/papers/10.1097-MD.0000000000036521.md</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="L43" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1097-MD.0000000000036521.md (../sources/papers/10.1097-MD.0000000000036521.md)</t>
+          <t>sources/papers/10.1097-MD.0000000000036521.md</t>
         </is>
       </c>
     </row>
@@ -3165,7 +3165,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1097-MD.0000000000036521.md (../sources/papers/10.1097-MD.0000000000036521.md)</t>
+          <t>sources/papers/10.1097-MD.0000000000036521.md</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2026.02.034.md (../sources/papers/10.1016-j.kint.2026.02.034.md)</t>
+          <t>sources/papers/10.1016-j.kint.2026.02.034.md</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2024.11.007.md (../sources/papers/10.1016-j.ekir.2024.11.007.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2024.11.007.md</t>
         </is>
       </c>
     </row>
@@ -3351,7 +3351,7 @@
       </c>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s10238-024-01461-6.md (../sources/papers/10.1007-s10238-024-01461-6.md)</t>
+          <t>sources/papers/10.1007-s10238-024-01461-6.md</t>
         </is>
       </c>
     </row>
@@ -3413,7 +3413,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.molimm.2022.01.011.md (../sources/papers/10.1016-j.molimm.2022.01.011.md)</t>
+          <t>sources/papers/10.1016-j.molimm.2022.01.011.md</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.3390-ijms241713063.md (../sources/papers/10.3390-ijms241713063.md)</t>
+          <t>sources/papers/10.3390-ijms241713063.md</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.3390-diagnostics13101729.md (../sources/papers/10.3390-diagnostics13101729.md)</t>
+          <t>sources/papers/10.3390-diagnostics13101729.md</t>
         </is>
       </c>
     </row>
@@ -3599,7 +3599,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.4049-jimmunol.2100924.md (../sources/papers/10.4049-jimmunol.2100924.md)</t>
+          <t>sources/papers/10.4049-jimmunol.2100924.md</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>mRNA levels of IL-6R, gp130, and STAT3 were significantly upregulated in PBMCs from IgAN patients vs. controls. In mice, DIO treatment visibly reduced mesangial IgA deposition, mesangial proliferation/matrix expansion, and Peyer's-patch lymphocyte hyperplasia, and suppressed p-JAK2/p-STAT3/STAT3 in Peyer's patches (n=6/group; qualitative/IHC endpoints, no group-level p-values given for histology). In DAKIKI cells, IL-6 (25 ng/mL) increased Gd-IgA1/IgA secretion and downregulated C1GalT1/Cosmc; DIO (1.0 µg/mL) dose-dependently suppressed IL-6-induced proliferation, IgA/Gd-IgA1 secretion (20.8% suppression at 1.0 µg/mL), JAK2/STAT3 mRNA upregulation, and STAT3 phosphorylation (significance denoted *p&lt;0.05/p&lt;0.01/*p&lt;0.001; exact p-values beyond these thresholds not extractable from available text).</t>
+          <t>mRNA levels of IL-6R, gp130, and STAT3 were significantly upregulated in PBMCs from IgAN patients vs. controls. In mice, DIO treatment visibly reduced mesangial IgA deposition, mesangial proliferation/matrix expansion, and Peyer's-patch lymphocyte hyperplasia, and suppressed p-JAK2/p-STAT3/STAT3 in Peyer's patches (n=6/group; qualitative/IHC endpoints, no group-level p-values given for histology). In DAKIKI cells, IL-6 (25 ng/mL) increased Gd-IgA1/IgA secretion and downregulated C1GalT1/Cosmc; DIO (1.0 µg/mL) dose-dependently suppressed IL-6-induced proliferation, IgA/Gd-IgA1 secretion (20.8% suppression at 1.0 µg/mL), JAK2/STAT3 mRNA upregulation, and STAT3 phosphorylation (significance denoted p&lt;0.05/p&lt;0.01/p&lt;0.001; exact p-values beyond these thresholds not extractable from available text).</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1186-s12882-025-04614-1.md (../sources/papers/10.1186-s12882-025-04614-1.md)</t>
+          <t>sources/papers/10.1186-s12882-025-04614-1.md</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s12026-025-09669-8.md (../sources/papers/10.1007-s12026-025-09669-8.md)</t>
+          <t>sources/papers/10.1007-s12026-025-09669-8.md</t>
         </is>
       </c>
     </row>
@@ -3770,7 +3770,7 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>Model validation: mesangial IgA deposition confirmed by IHC, significantly higher in IgAN group vs. control/SAR (p&lt;0.0001); SAR markedly attenuated IgA accumulation in IgAN+SAR (exact % values presented only graphically in figures, not printed in text). Renal function/proteinuria: urinary protein rose progressively in IgAN, peaking week 10; SAR significantly reduced proteinuria at weeks 10 and 12; serum urea/creatinine significantly higher in IgAN vs. control/SAR, significantly reduced by SAR (not fully normalized to healthy levels); SAR alone had no effect on renal parameters in healthy animals (exact numeric values/p-values for these panels given only as significance bands in figure legends: *p&lt;0.05 to p&lt;0.0001, not as printed values in running text). Inflammation/fibrosis markers: serum IL-6 significantly elevated in IgAN, significantly reduced by SAR; serum TNF-α showed only modest, apparently non-significant differences across groups; TGF-β1, SMAD3, and PDGF significantly elevated in IgAN vs. healthy groups, attenuated by SAR (most pronounced for TGF-β1/SMAD3); glomerular fibronectin and α-SMA (IHC) significantly increased in IgAN, significantly reduced by SAR though remaining above healthy levels. Masson's trichrome showed no significant collagen deposition in any group — authors interpret this as early fibrogenic activation preceding overt fibrosis, not established fibrosis. Oxford MEST-C: IgAN group had significantly higher frequencies of M1, E1, S1, T1, and C1 vs. control/SAR (Fisher's exact, *p&lt;0.05/*p&lt;0.001); SAR significantly reduced M1 and E1 prevalence specifically (from 100% in untreated IgAN to 28.6% in IgAN+SAR); reductions in S1, T1, and C1 with SAR were smaller and, per the authors' own discussion, non-significant. Podocyte integrity: TEM showed focal foot-process effacement in IgAN, partially preserved architecture in IgAN+SAR; nephrin and podocin (IHC and Western blot) significantly reduced in IgAN, significantly increased by SAR (partial restoration, remaining below healthy-group levels). No mortality in any group.</t>
+          <t>Model validation: mesangial IgA deposition confirmed by IHC, significantly higher in IgAN group vs. control/SAR (p&lt;0.0001); SAR markedly attenuated IgA accumulation in IgAN+SAR (exact % values presented only graphically in figures, not printed in text). Renal function/proteinuria: urinary protein rose progressively in IgAN, peaking week 10; SAR significantly reduced proteinuria at weeks 10 and 12; serum urea/creatinine significantly higher in IgAN vs. control/SAR, significantly reduced by SAR (not fully normalized to healthy levels); SAR alone had no effect on renal parameters in healthy animals (exact numeric values/p-values for these panels given only as significance bands in figure legends: p&lt;0.05 to p&lt;0.0001, not as printed values in running text). Inflammation/fibrosis markers: serum IL-6 significantly elevated in IgAN, significantly reduced by SAR; serum TNF-α showed only modest, apparently non-significant differences across groups; TGF-β1, SMAD3, and PDGF significantly elevated in IgAN vs. healthy groups, attenuated by SAR (most pronounced for TGF-β1/SMAD3); glomerular fibronectin and α-SMA (IHC) significantly increased in IgAN, significantly reduced by SAR though remaining above healthy levels. Masson's trichrome showed no significant collagen deposition in any group — authors interpret this as early fibrogenic activation preceding overt fibrosis, not established fibrosis. Oxford MEST-C: IgAN group had significantly higher frequencies of M1, E1, S1, T1, and C1 vs. control/SAR (Fisher's exact, p&lt;0.05/p&lt;0.001); SAR significantly reduced M1 and E1 prevalence specifically (from 100% in untreated IgAN to 28.6% in IgAN+SAR); reductions in S1, T1, and C1 with SAR were smaller and, per the authors' own discussion, non-significant. Podocyte integrity: TEM showed focal foot-process effacement in IgAN, partially preserved architecture in IgAN+SAR; nephrin and podocin (IHC and Western blot) significantly reduced in IgAN, significantly increased by SAR (partial restoration, remaining below healthy-group levels). No mortality in any group.</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1096-fj.202602487R.md (../sources/papers/10.1096-fj.202602487R.md)</t>
+          <t>sources/papers/10.1096-fj.202602487R.md</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.5414-CN111934.md (../sources/papers/10.5414-CN111934.md)</t>
+          <t>sources/papers/10.5414-CN111934.md</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1136-bmjopen-2026-120567.md (../sources/papers/10.1136-bmjopen-2026-120567.md)</t>
+          <t>sources/papers/10.1136-bmjopen-2026-120567.md</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1155-crin-7021133.md (../sources/papers/10.1155-crin-7021133.md)</t>
+          <t>sources/papers/10.1155-crin-7021133.md</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.2147-IJNRD.S631443.md (../sources/papers/10.2147-IJNRD.S631443.md)</t>
+          <t>sources/papers/10.2147-IJNRD.S631443.md</t>
         </is>
       </c>
     </row>
@@ -4095,7 +4095,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1038-s41584-026-01420-3.md (../sources/papers/10.1038-s41584-026-01420-3.md)</t>
+          <t>sources/papers/10.1038-s41584-026-01420-3.md</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2025.07.038.md (../sources/papers/10.1016-j.kint.2025.07.038.md)</t>
+          <t>sources/papers/10.1016-j.kint.2025.07.038.md</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2025.07.038.md (../sources/papers/10.1016-j.kint.2025.07.038.md)</t>
+          <t>sources/papers/10.1016-j.kint.2025.07.038.md</t>
         </is>
       </c>
     </row>
@@ -4281,7 +4281,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s11255-026-05103-6.md (../sources/papers/10.1007-s11255-026-05103-6.md)</t>
+          <t>sources/papers/10.1007-s11255-026-05103-6.md</t>
         </is>
       </c>
     </row>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.ekir.2026.106708.md (../sources/papers/10.1016-j.ekir.2026.106708.md)</t>
+          <t>sources/papers/10.1016-j.ekir.2026.106708.md</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.5414-CN112036.md (../sources/papers/10.5414-CN112036.md)</t>
+          <t>sources/papers/10.5414-CN112036.md</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4467,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.intimp.2026.117087.md (../sources/papers/10.1016-j.intimp.2026.117087.md)</t>
+          <t>sources/papers/10.1016-j.intimp.2026.117087.md</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-026-07337-z.md (../sources/papers/10.1007-s00467-026-07337-z.md)</t>
+          <t>sources/papers/10.1007-s00467-026-07337-z.md</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4591,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.7759-cureus.116913.md (../sources/papers/10.7759-cureus.116913.md)</t>
+          <t>sources/papers/10.7759-cureus.116913.md</t>
         </is>
       </c>
     </row>
@@ -4653,7 +4653,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.2169-internalmedicine.6751-25.md (../sources/papers/10.2169-internalmedicine.6751-25.md)</t>
+          <t>sources/papers/10.2169-internalmedicine.6751-25.md</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1080-0886022X.2026.2732704.md (../sources/papers/10.1080-0886022X.2026.2732704.md)</t>
+          <t>sources/papers/10.1080-0886022X.2026.2732704.md</t>
         </is>
       </c>
     </row>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.jprot.2026.105737.md (../sources/papers/10.1016-j.jprot.2026.105737.md)</t>
+          <t>sources/papers/10.1016-j.jprot.2026.105737.md</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,131 @@
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1136-bcr-2026-275498.md (../sources/papers/10.1136-bcr-2026-275498.md)</t>
+          <t>sources/papers/10.1136-bcr-2026-275498.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Rath et al. 2026</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Journal of Nephrology</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review and meta-analysis (tier 1)</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>9 retrospective cohorts, 1,185 kidney transplant recipients with recurrent/transplant IgA nephropathy (allograft-recurrence population — distinct from the native-kidney IgAN population in row 3 and the IgAV-nephritis population in row 39)</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>Oxford MEST-C classification components (M, E, S, T, C) and total MEST-C score, scored on allograft biopsies</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>None (prognostic/observational meta-analysis; univariable and multivariable HRs for graft loss pooled across cohorts via random-effects model)</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>S, T, and C lesions were consistently associated with allograft loss across pooled analyses; M and E lesions, and the total MEST-C score, showed inconsistent/non-independent associations in multivariable pooling. The total MEST-C score had univariable predictive value, but multivariable pooling did not confirm an independent association with graft loss. Subgroup/meta-regression identified geographic region, donor source, and cohort size as effect modifiers, explicitly described by the authors as exploratory/hypothesis-generating given the limited number of studies. Specific pooled HRs/CIs/p-values per MEST-C component were not reported in the abstract/metadata text available to this review and the full text is subscriber-only (Oxford Academic advance article) — marked "not extractable from available text."</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Tier 1 on the study-type ladder, but all 9 pooled cohorts are themselves retrospective; authors explicitly note heterogeneous study-specific multivariable models and a limited number of included studies as limitations, and state (quoted) that the total MEST-C score's "clinical utility requires robust prospective validation before routine reporting can be recommended." Independent reviewer assessment: the available abstract/metadata text did not report a formal risk-of-bias tool (e.g., ROBINS-I, QUIPS) applied to component cohorts, nor a funnel-plot/publication-bias assessment, nor funding/COI disclosures — all marked "not extractable from available text" (full text paywalled). Population distinction (per task instruction): this is a kidney-transplant/allograft-recurrence population, mechanistically and clinically distinct from native-kidney IgAN (row 3, Ștefan et al. 2023 — complement-pathway/MEST-C crescent association) and from IgAV-nephritis (row 39, Barbour et al. 2024 — only E1 independently prognostic for eGFR-decline trajectory); per research-question.md's topic-specific constraint, these findings are not merged. Noted pattern, not resolved: each of these three MEST-C studies finds a different component subset to be the "robust" prognostic one in its own population (crescents/complement in native IgAN; E1 alone in IgAV-N; S/T/C in transplant IgAN) — recorded as an observed cross-population pattern for research-writer/orchestrator awareness, not adjudicated here since the populations and outcomes differ.</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>10.1093/joneph/aajag258 / PMID 42874071</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1093-joneph.aajag258.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Yoo et al. 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>American Journal of Nephrology</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>Multicenter retrospective cohort with a defined comparator/reference group (tier 4)</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>788 adults with biopsy-proven IgAN, diagnosed 2002–2021; median follow-up 70 months</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>Hemoglobin level at biopsy, categorized into 5 bands (&lt;11.0, 11.0–11.9, 12.0–12.9 [reference], 13.0–13.9, ≥14.0 g/dL); sex-stratified analysis</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Reference band: Hb 12.0–12.9 g/dL</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>Primary outcome progression to ESKD: 66/788 (8.4%) progressed over median 70-month follow-up. Overall: Hb &lt;11.0 g/dL independently associated with higher ESKD risk vs. reference (aHR 2.88, 95% CI 1.24–6.68, p=0.014); restricted cubic spline showed a nonlinear relationship with risk rising markedly below ~12 g/dL. Sex-stratified: in women, Hb &lt;11.0 g/dL aHR 5.10 (95% CI 1.35–19.29, p=0.016) and Hb 11.0–11.9 g/dL aHR 4.66 (95% CI 1.26–17.19, p=0.021) were both significant; in men, no significant association was found (abstract reports no point estimates for the male stratum — marked "not extractable from available text"). Lower Hb was also associated with more severe tubular atrophy/interstitial fibrosis and endocapillary hypercellularity on biopsy (quantitative detail not given in the abstract — "not extractable from available text"). Authors conclude Hb may serve as (quoted) "a simple and clinically useful prognostic marker" for risk stratification in IgAN.</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Tier 4 (retrospective cohort with a defined comparator/reference band); multicenter design is a methodological strength. Standard retrospective-cohort limitations apply (no randomization; residual confounding). Authors' own stated limitations and funding/COI disclosures were not extractable from the abstract/metadata text available (full text subscriber-only, Karger "Subscribers Only") — marked "not extractable from available text." Independent reviewer-identified limitations: (1) possible reverse causation/residual confounding, since anemia severity is itself partly a consequence of CKD stage, and the abstract does not specify which covariates (e.g., baseline eGFR, proteinuria) were entered into the Cox models, so the degree of confounding control cannot be assessed from the available text; (2) the sex-stratified subgroup analysis (particularly the male stratum) may be underpowered given only 66 total ESKD events split across 2 sexes and 5 Hb bands — a null finding in men should not be read as equivalence without the (unreported) confidence intervals; (3) the long diagnosis window (2002–2021) raises a possible era effect (changes in background RAAS-blockade/SGLT2i therapy over two decades) not addressed in the available text.</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>10.1159/ajn/ablag012 / PMID 42858269</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>sources/papers/10.1159-ajn.ablag012.md</t>
         </is>
       </c>
     </row>
@@ -4857,13 +4981,13 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4936,7 +5060,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1038-s41581-024-00885-3.md (../sources/papers/10.1038-s41581-024-00885-3.md)</t>
+          <t>sources/papers/10.1038-s41581-024-00885-3.md</t>
         </is>
       </c>
     </row>
@@ -4973,7 +5097,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1038-s41572-023-00476-9.md (../sources/papers/10.1038-s41572-023-00476-9.md)</t>
+          <t>sources/papers/10.1038-s41572-023-00476-9.md</t>
         </is>
       </c>
     </row>
@@ -5010,7 +5134,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1016-j.kint.2023.04.029.md (../sources/papers/10.1016-j.kint.2023.04.029.md)</t>
+          <t>sources/papers/10.1016-j.kint.2023.04.029.md</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5171,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.3390-jcm13216621.md (../sources/papers/10.3390-jcm13216621.md)</t>
+          <t>sources/papers/10.3390-jcm13216621.md</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5208,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s10067-023-06781-8.md (../sources/papers/10.1007-s10067-023-06781-8.md)</t>
+          <t>sources/papers/10.1007-s10067-023-06781-8.md</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5245,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00467-026-07166-0.md (../sources/papers/10.1007-s00467-026-07166-0.md)</t>
+          <t>sources/papers/10.1007-s00467-026-07166-0.md</t>
         </is>
       </c>
     </row>
@@ -5158,7 +5282,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s00296-026-06295-x.md (../sources/papers/10.1007-s00296-026-06295-x.md)</t>
+          <t>sources/papers/10.1007-s00296-026-06295-x.md</t>
         </is>
       </c>
     </row>
@@ -5176,10 +5300,10 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5222,7 +5346,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/unverified-wadhwani-2024-jasn-pro-protect.md (../sources/papers/unverified-wadhwani-2024-jasn-pro-protect.md)</t>
+          <t>sources/papers/unverified-wadhwani-2024-jasn-pro-protect.md</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5368,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1136-bcr-2026-275354.md (../sources/papers/10.1136-bcr-2026-275354.md)</t>
+          <t>sources/papers/10.1136-bcr-2026-275354.md</t>
         </is>
       </c>
     </row>
@@ -5266,7 +5390,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>sources/papers/10.1007-s11255-026-05421-9.md (../sources/papers/10.1007-s11255-026-05421-9.md)</t>
+          <t>sources/papers/10.1007-s11255-026-05421-9.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regenerate exports with the weekly batch (rows 73-74)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrMqQ7Jh9rqNCt2Tcn7z5x
</commit_message>
<xml_diff>
--- a/outputs/evidence-table.xlsx
+++ b/outputs/evidence-table.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4964,6 +4964,130 @@
       <c r="L73" s="2" t="inlineStr">
         <is>
           <t>sources/papers/10.1159-ajn.ablag012.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Yoshida et al. 2026</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>The Journal of Dermatology</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Cross-sectional case-control mechanistic/biomarker study (tier 6 — pathogenesis-elucidating case-control, per judgment call #15 precedent)</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Human patients with IgA vasculitis (IgAV); serum analysis n=21 IgAV patients vs. 18 healthy donors; skin-biopsy immunofluorescence/in-situ-zymography subset n=11 IgAV patients (vs. control skin)</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>Serum anti-nephritis-associated-plasmin-receptor (anti-NAPlr) antibodies (IgG, IgM, IgA) by ELISA; skin-lesion NAPlr/plasmin-activity staining by immunofluorescence and in-situ zymography; serum galactose-deficient IgA1 (Gd-IgA1)</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Healthy donors (n=18) for serum ELISA; control (non-lesional/healthy) skin for histology</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Positive NAPlr/plasmin-activity staining observed in dermal lesions in 7/11 IgAV patients, vs. minimal staining in control skin. Serum anti-NAPlr IgG and IgA significantly elevated in IgAV vs. healthy donors (specific p-values not given in abstract — "not extractable from available text"). Anti-NAPlr IgG positively correlated with serum creatinine and negatively correlated with CH50, with a nonsignificant inverse association with eGFR. Serum Gd-IgA1 significantly increased in IgAV vs. controls, and positively correlated with anti-NAPlr IgA but negatively correlated with C4. Authors conclude these findings suggest an immune response to streptococcal NAPlr may contribute to IgA-mediated vascular inflammation, potentially through complement activation — relevant to the mucosal-immunity/infectious-trigger pathogenesis sub-topic (complements the background-context Filippatos et al. 2026 infectious-triggers review in the Background/Context table).</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Not applicable (cross-sectional design, single time-point sampling).</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>Full text was not obtainable: `mcp__PubMed__get_full_text_article` returned no PMC record, and `WebFetch` on the Wiley Online Library landing page returned HTTP 403 (paywalled); this is therefore an abstract/metadata-level extraction. Authors' own stated limitations, exact correlation coefficients/p-values, funding source, and conflict-of-interest disclosures were not given in the abstract and are marked "not extractable from available text." Independent reviewer-identified limitations: small sample size (n=21 vs. 18; histology subset n=11); cross-sectional design precludes causal/temporal inference about whether the anti-NAPlr antibody response precedes, coincides with, or follows renal involvement; single-center (Japan) — generalizability to other populations/streptococcal strain prevalence not established; correlation with creatinine/CH50 does not establish that NAPlr is causally nephritogenic in IgAV (as opposed to an epiphenomenon of a broader infection-triggered immune activation); no information on disease activity staging, treatment status at sampling, or exclusion of concurrent infection at the time of serum draw was extractable from the abstract.</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>10.1111/1346-8138.70548 / PMID 42907140</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Guzzo et al. 2026</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Journal of Nephrology</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>Retrospective cohort study + systematic literature review and meta-analysis of observational studies (tier 1 overall design, incorporating the authors' own tier-4 single-center retrospective cohort as one of the 6 pooled cohorts)</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Lausanne University Hospital retrospective cohort: 63 adult kidney-transplant recipients with biopsy-confirmed native-kidney IgAN (transplanted 2003–2019; of 97 IgAN transplant recipients, 34 excluded). Meta-analysis: 6 pooled cohorts (Stack 2000 Ireland n=42; Mousson 2007 France n=42; Avasare 2017 USA n=62; Garnier 2018 France n=67; Vasconcelos 2023 Brazil n=35 [native-biopsy data available for 35/53]; Lausanne 2025/2026 Switzerland n=63), total n=311, 23% with recurrent IgAN overall; crescent prevalence ranged 12–62% across cohorts</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>Presence/grade of glomerular crescents on the native (pre-transplant) kidney biopsy (Lausanne cohort scored via modified Oxford MEST-C: C0 none, C1 &lt;25% of viable glomeruli, C2 ≥25%; 8 patients without active crescents had fibrous crescents only; heterogeneous crescent definitions across the other 5 pooled cohorts)</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Patients without crescents, or with lower crescent grade, on native biopsy</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>Lausanne cohort: no significant association between native-kidney crescents and IgAN recurrence in the renal allograft (14/63 = 22.2% recurrence overall post-transplant; median follow-up 7.4 years, IQR 3.5–10.9; no significant differences in transplant characteristics/outcomes by crescent status). Meta-analysis of all 6 pooled cohorts (n=311): pooled RR for recurrence 1.53 (95% CI 0.40–5.90, p=.41) — confirms absence of association between native-kidney crescents and IgAN recurrence after transplantation, despite moderate heterogeneity (I²=72.09%, p=.02; Hartung-Knapp-Sidik-Jonkman adjustment method). Subgroup of the 3 cohorts using a MEST-C-based crescent definition (Avasare, Vasconcelos, Lausanne) showed the same null association. Meta-regression on cohort publication year suggested era-related confounding within the C1 and C2 subgroups specifically (p=.01 and p=.008) but not in a meta-regression on the full pooled set (p=.29). Authors conclude: glomerular crescents — especially when present in ≥25% of viable glomeruli — remain an unfavorable prognostic factor for progression of NATIVE-kidney IgAN to kidney failure, but do not appear to represent a risk factor for IgAN disease recurrence in the renal allograft after transplantation. Population/outcome distinction (per task instruction, not resolved by this reviewer): this null finding concerns native-kidney crescents predicting allograft disease recurrence (recurrent IgA deposits on transplant biopsy); it addresses a related but distinct question from row 71 (Rath et al. 2026), which found that S/T/C MEST-C lesions scored on the allograft biopsy itself (in an already-transplanted/recurrent-IgAN population) DO predict allograft loss (a structural/functional graft-survival endpoint, any cause). The two findings sit in overlapping but non-identical transplant-IgAN populations and measure different exposures (native pre-transplant biopsy vs. allograft biopsy) and different outcomes (recurrence vs. graft loss) — this is flagged as a non-contradictory pattern worth distinguishing in synthesis, not a conflict to adjudicate.</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Lausanne cohort median post-transplant follow-up 7.4 years (IQR 3.5–10.9), outcome ascertained at last visit, graft failure, or 31 December 2022.</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>Authors' stated limitations (quoted/paraphrased from full text): retrospective design with possible selection bias and incomplete historical data; unusually high crescent prevalence across the pooled cohorts, which may reduce discriminatory power; small sample sizes, so the overall analysis may be underpowered — authors explicitly state the null result may reflect low statistical power rather than a true absence of association; heterogeneous crescent definitions across the 6 cohorts; possible confounding by changes in immunosuppression protocols over the two-decade+ study span; possible publication bias (Egger's test p=.08, though trim-and-fill did not substantially change the pooled estimate); only 6 cohorts included, with low-to-moderate methodological quality (Newcastle-Ottawa scores 5–7), and reliance on a single summary statistic per cohort. Funding: authors state the work received no financial support from pharmaceutical companies or other commercial entities; no specific funder named. Conflicts of interest: authors declare none. Independent reviewer-identified limitations: native-biopsy timing relative to transplantation, and each center's surveillance- vs. for-cause-biopsy protocol for detecting recurrence, are not reported in a way that allows assessment of whether detection sensitivity for "recurrence" was comparable across the 6 different centers/eras (2000–2026); the wide confidence interval (0.40–5.90) around the pooled RR means a clinically meaningful association cannot be confidently excluded, consistent with the authors' own power concern.</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>10.1093/joneph/aajag169 / PMID 42696417</t>
         </is>
       </c>
     </row>

</xml_diff>